<commit_message>
Supply map rebuilt on original branded template; Emblem promoted to proposed row #44
- Map: Milestone-branded template (navy header, magenta subject star, gold ring),
  47 numbered pins with CoStar-exact coords where available, purple shadow +
  gray documented-dead pins
- Chart: Emblem Meridian added as #44 (250u, TBD, Bear-only toggle); proposed
  section now 15 properties / 3,942 units; forecast ranges extended

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CQcHG3mGNNEuNdk4jQMCJB
</commit_message>
<xml_diff>
--- a/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
+++ b/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
@@ -217,7 +217,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -240,11 +240,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -456,6 +500,8 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -847,7 +893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:M60"/>
+  <dimension ref="A2:M61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="79" min="1" max="1"/>
@@ -2374,7 +2420,7 @@
       <c r="B43" s="23" t="n"/>
       <c r="C43" s="83" t="inlineStr">
         <is>
-          <t>PROPOSED (14 properties, 3,692 units)</t>
+          <t>PROPOSED (15 properties, 3,942 units)</t>
         </is>
       </c>
     </row>
@@ -2874,11 +2920,11 @@
       </c>
       <c r="C55" s="25" t="inlineStr">
         <is>
-          <t>12548 West Overland Road</t>
+          <t>Emblem Meridian (Quarterra)</t>
         </is>
       </c>
       <c r="D55" s="26" t="n">
-        <v>156</v>
+        <v>250</v>
       </c>
       <c r="E55" s="24" t="inlineStr">
         <is>
@@ -2893,20 +2939,20 @@
       </c>
       <c r="H55" s="25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Quarterra</t>
         </is>
       </c>
       <c r="I55" s="29" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="J55" s="24" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K55" s="25" t="inlineStr">
         <is>
-          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed - stalled; PUD likely lapsed ~Mar 2026 - RV storage still operating</t>
+          <t>Analyst-sourced (not in CoStar/RealPage); Diligence: proposed - formal early plans filed June 2026; 250u (apts+TH) on ~13 ac R-15, N of Eagle &amp; Victory; ex-Artisan Victory Market site; nearest live MF application to subject</t>
         </is>
       </c>
       <c r="M55">
@@ -2920,11 +2966,11 @@
       </c>
       <c r="C56" s="25" t="inlineStr">
         <is>
-          <t>Ascent Overland</t>
+          <t>12548 West Overland Road</t>
         </is>
       </c>
       <c r="D56" s="26" t="n">
-        <v>138</v>
+        <v>156</v>
       </c>
       <c r="E56" s="24" t="inlineStr">
         <is>
@@ -2943,7 +2989,7 @@
         </is>
       </c>
       <c r="I56" s="29" t="n">
-        <v>1.5</v>
+        <v>1.1</v>
       </c>
       <c r="J56" s="24" t="inlineStr">
         <is>
@@ -2952,7 +2998,7 @@
       </c>
       <c r="K56" s="25" t="inlineStr">
         <is>
-          <t>Diligence: proposed - stalled; entitled site for sale via CBRE at $5.0M</t>
+          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed - stalled; PUD likely lapsed ~Mar 2026 - RV storage still operating</t>
         </is>
       </c>
       <c r="M56">
@@ -2966,11 +3012,11 @@
       </c>
       <c r="C57" s="25" t="inlineStr">
         <is>
-          <t>Meridian OZ Apartments</t>
+          <t>Ascent Overland</t>
         </is>
       </c>
       <c r="D57" s="26" t="n">
-        <v>36</v>
+        <v>138</v>
       </c>
       <c r="E57" s="24" t="inlineStr">
         <is>
@@ -2985,20 +3031,20 @@
       </c>
       <c r="H57" s="25" t="inlineStr">
         <is>
-          <t>Peak Capital Investments Llc</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I57" s="29" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="J57" s="24" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K57" s="25" t="inlineStr">
         <is>
-          <t>Diligence: proposed - stalled; downsized to 36u Oct 2024 - entitled site listed then off-market</t>
+          <t>Diligence: proposed - stalled; entitled site for sale via CBRE at $5.0M</t>
         </is>
       </c>
       <c r="M57">
@@ -3006,9 +3052,56 @@
         <v/>
       </c>
     </row>
+    <row r="58">
+      <c r="B58" s="24" t="n">
+        <v>47</v>
+      </c>
+      <c r="C58" s="25" t="inlineStr">
+        <is>
+          <t>Meridian OZ Apartments</t>
+        </is>
+      </c>
+      <c r="D58" s="26" t="n">
+        <v>36</v>
+      </c>
+      <c r="E58" s="24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F58" s="27" t="n"/>
+      <c r="G58" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H58" s="25" t="inlineStr">
+        <is>
+          <t>Peak Capital Investments Llc</t>
+        </is>
+      </c>
+      <c r="I58" s="29" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J58" s="24" t="inlineStr">
+        <is>
+          <t>Garden</t>
+        </is>
+      </c>
+      <c r="K58" s="25" t="inlineStr">
+        <is>
+          <t>Diligence: proposed - stalled; downsized to 36u Oct 2024 - entitled site listed then off-market</t>
+        </is>
+      </c>
+      <c r="M58">
+        <f>IFERROR(VALUE(RIGHT(E58,4))*4+MATCH(LEFT(E58,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
+      </c>
+    </row>
     <row r="59"/>
-    <row r="60">
-      <c r="B60" s="84" t="inlineStr">
+    <row r="60"/>
+    <row r="61">
+      <c r="B61" s="84" t="inlineStr">
         <is>
           <t>* 5-Mile radius. Rent ($) = HelloData mix-weighted asking where covered, else market asking (CoStar). Proximity (mi) = straight-line distance from the subject. Est. Delivery drives the Supply &amp; Absorption tab's per-window supply (edit it there or here — they are linked). See the 'Supply &amp; Absorption' tab for the forward supply / absorption / overall-occupancy forecast.</t>
         </is>
@@ -3034,7 +3127,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:Z75"/>
+  <dimension ref="A1:Z75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="1"/>
   <cols>
     <col width="2.44140625" customWidth="1" style="79" min="1" max="1"/>
@@ -3643,31 +3736,31 @@
         <v>450</v>
       </c>
       <c r="I19" s="46">
-        <f>SUMIFS('Competitive Analysis'!$D$5:$D$57,'Competitive Analysis'!$M$5:$M$57,"&gt;="&amp;8102,'Competitive Analysis'!$M$5:$M$57,"&lt;="&amp;8105)</f>
+        <f>SUMIFS('Competitive Analysis'!$D$5:$D$58,'Competitive Analysis'!$M$5:$M$58,"&gt;="&amp;8102,'Competitive Analysis'!$M$5:$M$58,"&lt;="&amp;8105)</f>
         <v/>
       </c>
       <c r="J19" s="47">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,1)+SUMIFS($S$13:$S$26,$W$13:$W$26,1,$X$13:$X$26,1)</f>
+        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,1)+SUMIFS($S$13:$S$27,$W$13:$W$27,1,$X$13:$X$27,1)</f>
         <v/>
       </c>
       <c r="K19" s="47">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,2)+SUMIFS($S$13:$S$26,$W$13:$W$26,2,$X$13:$X$26,1)</f>
+        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,2)+SUMIFS($S$13:$S$27,$W$13:$W$27,2,$X$13:$X$27,1)</f>
         <v/>
       </c>
       <c r="L19" s="47">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,3)+SUMIFS($S$13:$S$26,$W$13:$W$26,3,$X$13:$X$26,1)</f>
+        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,3)+SUMIFS($S$13:$S$27,$W$13:$W$27,3,$X$13:$X$27,1)</f>
         <v/>
       </c>
       <c r="M19" s="47">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,4)+SUMIFS($S$13:$S$26,$W$13:$W$26,4,$X$13:$X$26,1)</f>
+        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,4)+SUMIFS($S$13:$S$27,$W$13:$W$27,4,$X$13:$X$27,1)</f>
         <v/>
       </c>
       <c r="N19" s="47">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,5)+SUMIFS($S$13:$S$26,$W$13:$W$26,5,$X$13:$X$26,1)</f>
+        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,5)+SUMIFS($S$13:$S$27,$W$13:$W$27,5,$X$13:$X$27,1)</f>
         <v/>
       </c>
       <c r="O19" s="47">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,6)+SUMIFS($S$13:$S$26,$W$13:$W$26,6,$X$13:$X$26,1)</f>
+        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,6)+SUMIFS($S$13:$S$27,$W$13:$W$27,6,$X$13:$X$27,1)</f>
         <v/>
       </c>
       <c r="R19" s="37" t="inlineStr">
@@ -4249,6 +4342,36 @@
       </c>
       <c r="O27" s="56">
         <f>IFERROR('[1]Cash Flow (Annual)'!$P$14,"")</f>
+        <v/>
+      </c>
+      <c r="R27" s="37" t="inlineStr">
+        <is>
+          <t>Emblem Meridian (Quarterra)</t>
+        </is>
+      </c>
+      <c r="S27" s="38" t="n">
+        <v>250</v>
+      </c>
+      <c r="T27" s="43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="U27" s="43" t="inlineStr">
+        <is>
+          <t>Bear only</t>
+        </is>
+      </c>
+      <c r="V27">
+        <f>IFERROR(VALUE(RIGHT(T27,4))*4+MATCH(LEFT(T27,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
+      </c>
+      <c r="W27">
+        <f>IF(V27="","",IF(V27&lt;=$Z$1,0,MAX(1,INT((V27-$Z$2)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X27">
+        <f>IF(U27="All",1,IF(U27="Bear+Base",IF($Z$3&gt;=2,1,0),IF(U27="Bear only",IF($Z$3&gt;=3,1,0),0)))</f>
         <v/>
       </c>
     </row>
@@ -5330,7 +5453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P47"/>
+  <dimension ref="A1:P48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" customWidth="1" style="79" min="1" max="1"/>
@@ -7659,6 +7782,43 @@
       <c r="P47" t="inlineStr">
         <is>
           <t>Audit find Aug 2026 — promoted from shadow watch; Elk Ventures 516u CUP; groundbreaking expected 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Emblem Meridian (Quarterra)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2820 S Eagle Rd area, N of Eagle &amp; Victory</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>250</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+      <c r="H48" s="75" t="n"/>
+      <c r="I48" s="75" t="n"/>
+      <c r="J48" s="75" t="n"/>
+      <c r="K48" s="76" t="n"/>
+      <c r="L48" s="76" t="n"/>
+      <c r="M48" s="76" t="n"/>
+      <c r="N48" s="76" t="n"/>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Diligence</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Promoted from shadow watch Aug 2026 — formal early plans filed June 2026 (BoiseDev)</t>
         </is>
       </c>
     </row>
@@ -7673,7 +7833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H54"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="2.44140625" customWidth="1" style="79" min="1" max="1"/>
@@ -7686,6 +7846,7 @@
     <col width="36" customWidth="1" style="79" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="86" t="inlineStr">
         <is>
@@ -8529,36 +8690,19 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="B32" s="37" t="inlineStr">
         <is>
           <t>Outer Banks Apartments</t>
         </is>
       </c>
-      <c r="C32" s="77" t="n">
-        <v>516</v>
-      </c>
-      <c r="D32" s="77" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="E32" s="37" t="inlineStr">
-        <is>
-          <t>proposed - near-UC; groundbreaking expected 2026</t>
-        </is>
-      </c>
-      <c r="F32" s="37" t="n"/>
-      <c r="G32" s="37" t="inlineStr">
-        <is>
-          <t>AUG 2026 AUDIT: promoted from shadow watch. Elk Ventures CUP 2024: 516 units (364 apts, 126 flats, 26 TH) on 19.34 ac R-40/C-C, SW corner Franklin &amp; Ten Mile. Statesman 2026 outlook: groundbreaking expected 2026, 14-16 mo build, first units summer 2027. Was entitled 2021 as "Outer Banks Sub" — plat-style name, no apartment brand, hence invisible to feeds.</t>
-        </is>
-      </c>
-      <c r="H32" s="37" t="inlineStr">
-        <is>
-          <t>https://www.yahoo.com/news/articles/meridian-keeps-changing-see-key-110000519.html</t>
-        </is>
-      </c>
+      <c r="C32" s="87" t="n"/>
+      <c r="D32" s="87" t="n"/>
+      <c r="E32" s="87" t="n"/>
+      <c r="F32" s="87" t="n"/>
+      <c r="G32" s="87" t="n"/>
+      <c r="H32" s="88" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="37" t="inlineStr">
@@ -8588,83 +8732,89 @@
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="86" t="inlineStr">
+      <c r="B34" s="37" t="inlineStr">
+        <is>
+          <t>Emblem Meridian (Quarterra)</t>
+        </is>
+      </c>
+      <c r="C34" s="77" t="n">
+        <v>250</v>
+      </c>
+      <c r="D34" s="77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E34" s="37" t="inlineStr">
+        <is>
+          <t>proposed - formal early plans filed June 2026</t>
+        </is>
+      </c>
+      <c r="F34" s="37" t="n"/>
+      <c r="G34" s="37" t="inlineStr">
+        <is>
+          <t>PROMOTED from shadow watch Aug 2026 (user call: it is a live proposal). Quarterra "Emblem Meridian" 250 units (apartments + TH) on ~13 ac R-15, N of Eagle &amp; Victory — ex-Artisan Victory Market site (H-2022-0066 131u BTR approved 2023, never built). Formal early plans filed June 2026 per BoiseDev 6/10/26; no hearing date yet. Nearest live MF application to the subject (1.0 mi, same Eagle Rd corridor).</t>
+        </is>
+      </c>
+      <c r="H34" s="37" t="inlineStr">
+        <is>
+          <t>https://boisedev.com/news/2026/06/10/meridian-emblem-victory-eagle-homes-apartment/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="86" t="inlineStr">
         <is>
           <t>SHADOW SUPPLY (latent / untracked — watch list)</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="44" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="44" t="inlineStr">
         <is>
           <t>Property / Site</t>
         </is>
       </c>
-      <c r="C35" s="44" t="inlineStr">
+      <c r="C36" s="44" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="D35" s="44" t="inlineStr">
+      <c r="D36" s="44" t="inlineStr">
         <is>
           <t>Est. Delivery</t>
         </is>
       </c>
-      <c r="E35" s="44" t="inlineStr">
+      <c r="E36" s="44" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F35" s="44" t="inlineStr">
+      <c r="F36" s="44" t="inlineStr">
         <is>
           <t>Leasing Pace</t>
         </is>
       </c>
-      <c r="G35" s="44" t="inlineStr">
+      <c r="G36" s="44" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H35" s="44" t="inlineStr">
+      <c r="H36" s="44" t="inlineStr">
         <is>
           <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="37" t="inlineStr">
-        <is>
-          <t>Emblem Meridian (Quarterra) / Artisan Victory Market site</t>
-        </is>
-      </c>
-      <c r="C36" s="77" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
-      </c>
-      <c r="D36" s="77" t="n"/>
-      <c r="E36" s="37" t="n"/>
-      <c r="F36" s="37" t="n"/>
-      <c r="G36" s="37" t="inlineStr">
-        <is>
-          <t>Land-use analysis site SM-76: ~12-ac BPS Eagle Road LLC assemblage on S Eagle Rd. 'Artisan Victory Market' (H-2022-0066) approved 2023 for 131 build-to-rent units + commercial but never built; superseded by Quarterra's 'Emblem Meridian' ~250-unit concept (pre-application June 2026). Closest large latent MF site to the subject (~1 mi). | AUG 2026 AUDIT: formal early plans FILED June 2026 — 250 units (apts+TH) on ~13 ac (BoiseDev 6/10/26). Nearest live MF application to the subject (1.0 mi).</t>
-        </is>
-      </c>
-      <c r="H36" s="37" t="inlineStr">
-        <is>
-          <t>https://boisedev.com/news/2026/06/10/meridian-emblem-victory-eagle-homes-apartment/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="37" t="inlineStr">
         <is>
-          <t>Tanner Creek apartments (Waltman/Johnson Ln)</t>
+          <t>Emblem Meridian (Quarterra) / Artisan Victory Market site</t>
         </is>
       </c>
       <c r="C37" s="77" t="inlineStr">
         <is>
-          <t>280</t>
+          <t>250</t>
         </is>
       </c>
       <c r="D37" s="77" t="n"/>
@@ -8672,24 +8822,24 @@
       <c r="F37" s="37" t="n"/>
       <c r="G37" s="37" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-15: Tanner Creek (heard Nov 2023; moved forward) — 83 SF homes + 45 townhomes + 280 phased apartments on ~38 ac, paired with ~30-ac Hawkins commercial between I-84 and Waltman Ln. Residential now being built by CBH Homes; the 280-unit apartment component is latent supply not yet in the CoStar/RealPage pipeline.</t>
+          <t>PROMOTED Aug 2026 to pipeline row #44 (250u) — kept here for history. Land-use analysis site SM-76: ~12-ac BPS Eagle Road LLC assemblage on S Eagle Rd. 'Artisan Victory Market' (H-2022-0066) approved 2023 for 131 build-to-rent units + commercial but never built; superseded by Quarterra's 'Emblem Meridian' ~250-unit concept (pre-application June 2026). Closest large latent MF site to the subject (~1 mi). | AUG 2026 AUDIT: formal early plans FILED June 2026 — 250 units (apts+TH) on ~13 ac (BoiseDev 6/10/26). Nearest live MF application to the subject (1.0 mi).</t>
         </is>
       </c>
       <c r="H37" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2023/11/28/plans-for-two-large-developments-off-i-84-and-meridian-rd-move-forward/</t>
+          <t>https://boisedev.com/news/2026/06/10/meridian-emblem-victory-eagle-homes-apartment/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="37" t="inlineStr">
         <is>
-          <t>Graycliff Estates R-40 block</t>
+          <t>Tanner Creek apartments (Waltman/Johnson Ln)</t>
         </is>
       </c>
       <c r="C38" s="77" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>280</t>
         </is>
       </c>
       <c r="D38" s="77" t="n"/>
@@ -8697,40 +8847,44 @@
       <c r="F38" s="37" t="n"/>
       <c r="G38" s="37" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-3: Graycliff Estates (Star Development) approved preliminary plat of ~200 SF homes PLUS 224 apartments (R-40 high-density block) on ~52 ac; SF portion building since 2021. The 224-unit apartment block remains unbuilt latent supply. | AUG 2026 AUDIT: confirmed still unbuilt; no 2026 hearing/permit activity found.</t>
+          <t>Land-use analysis site SM-15: Tanner Creek (heard Nov 2023; moved forward) — 83 SF homes + 45 townhomes + 280 phased apartments on ~38 ac, paired with ~30-ac Hawkins commercial between I-84 and Waltman Ln. Residential now being built by CBH Homes; the 280-unit apartment component is latent supply not yet in the CoStar/RealPage pipeline.</t>
         </is>
       </c>
       <c r="H38" s="37" t="inlineStr">
         <is>
-          <t>https://www.weknowboise.com/graycliff-estates.php</t>
+          <t>https://boisedev.com/news/2023/11/28/plans-for-two-large-developments-off-i-84-and-meridian-rd-move-forward/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="37" t="inlineStr">
         <is>
-          <t>Touchmark Meadow Lake Village expansion</t>
-        </is>
-      </c>
-      <c r="C39" s="77" t="n"/>
+          <t>Graycliff Estates R-40 block</t>
+        </is>
+      </c>
+      <c r="C39" s="77" t="inlineStr">
+        <is>
+          <t>224</t>
+        </is>
+      </c>
       <c r="D39" s="77" t="n"/>
       <c r="E39" s="37" t="n"/>
       <c r="F39" s="37" t="n"/>
       <c r="G39" s="37" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-9: ~64 undeveloped ac of Touchmark's ~121-ac senior community. July 2025 development-modification agreement + rezone + PUD in progress to a broader 'Touchmark Mixed Use' (mixed housing types). Senior-oriented, but adds rental housing capacity 1.5 mi from subject.</t>
+          <t>Land-use analysis site SM-3: Graycliff Estates (Star Development) approved preliminary plat of ~200 SF homes PLUS 224 apartments (R-40 high-density block) on ~52 ac; SF portion building since 2021. The 224-unit apartment block remains unbuilt latent supply. | AUG 2026 AUDIT: confirmed still unbuilt; no 2026 hearing/permit activity found.</t>
         </is>
       </c>
       <c r="H39" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2025/07/14/touchmark-meridian-meadowlake-mixed-use/</t>
+          <t>https://www.weknowboise.com/graycliff-estates.php</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="37" t="inlineStr">
         <is>
-          <t>Ten Mile Crossing residual HDR parcels</t>
+          <t>Touchmark Meadow Lake Village expansion</t>
         </is>
       </c>
       <c r="C40" s="77" t="n"/>
@@ -8739,19 +8893,19 @@
       <c r="F40" s="37" t="n"/>
       <c r="G40" s="37" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-4: residential portion (R-15/R-8) of Brighton's Ten Mile Crossing at SW Overland &amp; Ten Mile — partially built (Cortland South Meridian + CBH SF); remaining High-Density Residential parcels planned/dormant, including an 8.6-ac and a 14.4-ac R-15 vacant parcel (highest-interest sites in the land-use ranking). Note: South Ridge II (164u UC, tracked in the chart) is rising in this same corridor.</t>
+          <t>Land-use analysis site SM-9: ~64 undeveloped ac of Touchmark's ~121-ac senior community. July 2025 development-modification agreement + rezone + PUD in progress to a broader 'Touchmark Mixed Use' (mixed housing types). Senior-oriented, but adds rental housing capacity 1.5 mi from subject.</t>
         </is>
       </c>
       <c r="H40" s="37" t="inlineStr">
         <is>
-          <t>https://www.brighton.co/brighton-place/ten-mile-crossing/</t>
+          <t>https://boisedev.com/news/2025/07/14/touchmark-meridian-meadowlake-mixed-use/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="37" t="inlineStr">
         <is>
-          <t>Brighton Apex R-15 parcel (Lake Hazel)</t>
+          <t>Ten Mile Crossing residual HDR parcels</t>
         </is>
       </c>
       <c r="C41" s="77" t="n"/>
@@ -8760,19 +8914,19 @@
       <c r="F41" s="37" t="n"/>
       <c r="G41" s="37" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-61: 15.1-ac R-15 (med-high-density) parcel on E Lake Hazel Rd inside Brighton's approved Apex/Pinnacle master-plan footprint; adjacent phases actively building. Latent MF-capable ground in the fast-growing S Meridian corridor.</t>
+          <t>Land-use analysis site SM-4: residential portion (R-15/R-8) of Brighton's Ten Mile Crossing at SW Overland &amp; Ten Mile — partially built (Cortland South Meridian + CBH SF); remaining High-Density Residential parcels planned/dormant, including an 8.6-ac and a 14.4-ac R-15 vacant parcel (highest-interest sites in the land-use ranking). Note: South Ridge II (164u UC, tracked in the chart) is rising in this same corridor.</t>
         </is>
       </c>
       <c r="H41" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2024/12/20/brighton-pinnacle-costco-meridian/</t>
+          <t>https://www.brighton.co/brighton-place/ten-mile-crossing/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="37" t="inlineStr">
         <is>
-          <t>Outer Banks Subdivision (TM Creek / Cobalt Dr)</t>
+          <t>Brighton Apex R-15 parcel (Lake Hazel)</t>
         </is>
       </c>
       <c r="C42" s="77" t="n"/>
@@ -8781,49 +8935,45 @@
       <c r="F42" s="37" t="n"/>
       <c r="G42" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROMOTED Aug 2026 to pipeline row #33 "Outer Banks Apartments" (516u, groundbreaking expected 2026) — kept here for history. </t>
+          <t>Land-use analysis site SM-61: 15.1-ac R-15 (med-high-density) parcel on E Lake Hazel Rd inside Brighton's approved Apex/Pinnacle master-plan footprint; adjacent phases actively building. Latent MF-capable ground in the fast-growing S Meridian corridor.</t>
         </is>
       </c>
       <c r="H42" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2021/12/17/outer-banks-pera-place/</t>
+          <t>https://boisedev.com/news/2024/12/20/brighton-pinnacle-costco-meridian/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="37" t="inlineStr">
         <is>
-          <t>Grandview Communities (Lake Hazel &amp; Linder)</t>
-        </is>
-      </c>
-      <c r="C43" s="77" t="inlineStr">
-        <is>
-          <t>130</t>
-        </is>
-      </c>
+          <t>Outer Banks Subdivision (TM Creek / Cobalt Dr)</t>
+        </is>
+      </c>
+      <c r="C43" s="77" t="n"/>
       <c r="D43" s="77" t="n"/>
       <c r="E43" s="37" t="n"/>
       <c r="F43" s="37" t="n"/>
       <c r="G43" s="37" t="inlineStr">
         <is>
-          <t>AUDIT WATCH: 79-ac pre-application (July 2025) at NE corner Lake Hazel &amp; Linder — ~510 homes incl. ~130 apartments + 176 TH/cluster; no formal H-file or hearing yet; sits near the southern ring edge (~4.5 mi).</t>
+          <t xml:space="preserve">PROMOTED Aug 2026 to pipeline row #33 "Outer Banks Apartments" (516u, groundbreaking expected 2026) — kept here for history. </t>
         </is>
       </c>
       <c r="H43" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2025/07/07/hundreds-of-homes-apartments-planned-for-lake-hazel-and-linder/</t>
+          <t>https://boisedev.com/news/2021/12/17/outer-banks-pera-place/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="37" t="inlineStr">
         <is>
-          <t>Discovery project (Lake Hazel &amp; Locust Grove)</t>
+          <t>Grandview Communities (Lake Hazel &amp; Linder)</t>
         </is>
       </c>
       <c r="C44" s="77" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>130</t>
         </is>
       </c>
       <c r="D44" s="77" t="n"/>
@@ -8831,40 +8981,44 @@
       <c r="F44" s="37" t="n"/>
       <c r="G44" s="37" t="inlineStr">
         <is>
-          <t>AUDIT WATCH: April 2024 pre-application for 200+ units (nine 3-story buildings + TH/SFR) on ~20 ac by Discovery Park; no formal application since — dormant but the land is teed up (~3.5 mi).</t>
+          <t>AUDIT WATCH: 79-ac pre-application (July 2025) at NE corner Lake Hazel &amp; Linder — ~510 homes incl. ~130 apartments + 176 TH/cluster; no formal H-file or hearing yet; sits near the southern ring edge (~4.5 mi).</t>
         </is>
       </c>
       <c r="H44" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2024/04/12/200-apartments-meridian-discovery/</t>
+          <t>https://boisedev.com/news/2025/07/07/hundreds-of-homes-apartments-planned-for-lake-hazel-and-linder/</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="37" t="inlineStr">
         <is>
-          <t>709 N Cole Rd (city land trust)</t>
-        </is>
-      </c>
-      <c r="C45" s="77" t="n"/>
+          <t>Discovery project (Lake Hazel &amp; Locust Grove)</t>
+        </is>
+      </c>
+      <c r="C45" s="77" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
       <c r="D45" s="77" t="n"/>
       <c r="E45" s="37" t="n"/>
       <c r="F45" s="37" t="n"/>
       <c r="G45" s="37" t="inlineStr">
         <is>
-          <t>AUDIT WATCH: City of Boise closing (July 2026) on 1.64 ac by Boise Towne Square for future affordable housing (prior owner proposed 71 micro-units in 2021); no developer or program yet — 2029+ speculative. Same parcel as the excluded 'Cole Road' RealPage entry.</t>
+          <t>AUDIT WATCH: April 2024 pre-application for 200+ units (nine 3-story buildings + TH/SFR) on ~20 ac by Discovery Park; no formal application since — dormant but the land is teed up (~3.5 mi).</t>
         </is>
       </c>
       <c r="H45" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2026/06/01/709-cole-boise/</t>
+          <t>https://boisedev.com/news/2024/04/12/200-apartments-meridian-discovery/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="37" t="inlineStr">
         <is>
-          <t>Aren east phase (verify)</t>
+          <t>709 N Cole Rd (city land trust)</t>
         </is>
       </c>
       <c r="C46" s="77" t="n"/>
@@ -8873,19 +9027,19 @@
       <c r="F46" s="37" t="n"/>
       <c r="G46" s="37" t="inlineStr">
         <is>
-          <t>AUDIT WATCH: The Aren (396u, delivered 2024) was planned as two phases at Eagle View Landing; verify whether the east-phase (~200u) buildings are fully delivered within the tracked 396 or represent additional untracked pipeline.</t>
+          <t>AUDIT WATCH: City of Boise closing (July 2026) on 1.64 ac by Boise Towne Square for future affordable housing (prior owner proposed 71 micro-units in 2021); no developer or program yet — 2029+ speculative. Same parcel as the excluded 'Cole Road' RealPage entry.</t>
         </is>
       </c>
       <c r="H46" s="37" t="inlineStr">
         <is>
-          <t>https://arenmeridian.com/</t>
+          <t>https://boisedev.com/news/2026/06/01/709-cole-boise/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="37" t="inlineStr">
         <is>
-          <t>Murio Farms MF phases (SW Boise)</t>
+          <t>Aren east phase (verify)</t>
         </is>
       </c>
       <c r="C47" s="77" t="n"/>
@@ -8894,109 +9048,109 @@
       <c r="F47" s="37" t="n"/>
       <c r="G47" s="37" t="inlineStr">
         <is>
-          <t>AUDIT WATCH: 380-ac, 3,500-home master plan approved 2024 between Maple Grove &amp; Cole at the New York Canal; apartments in later phases (15-20 yr buildout) — long-dated only.</t>
+          <t>AUDIT WATCH: The Aren (396u, delivered 2024) was planned as two phases at Eagle View Landing; verify whether the east-phase (~200u) buildings are fully delivered within the tracked 396 or represent additional untracked pipeline.</t>
         </is>
       </c>
       <c r="H47" s="37" t="inlineStr">
         <is>
-          <t>https://www.ktvb.com/article/news/local/idaho-press/city-council-approves-murio-farms-3500-homes-southwest-boise/277-eb746dad-15bb-4c8e-868d-ca9d6c1e355e</t>
+          <t>https://arenmeridian.com/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="37" t="inlineStr">
         <is>
-          <t>Pine 43 VI residential (same MDA as the 270u CUP)</t>
-        </is>
-      </c>
-      <c r="C48" s="77" t="n">
-        <v>604</v>
-      </c>
+          <t>Murio Farms MF phases (SW Boise)</t>
+        </is>
+      </c>
+      <c r="C48" s="77" t="n"/>
       <c r="D48" s="77" t="n"/>
       <c r="E48" s="37" t="n"/>
       <c r="F48" s="37" t="n"/>
       <c r="G48" s="37" t="inlineStr">
         <is>
-          <t>AUG 2026 AUDIT: H-2024-0071 (approved 10/21/2025) also allows up to 604 vertically-integrated units over ground-floor commercial (87-ft height exception) + 30 TH — up to 904 total units in the Pine 43 revamp (~$1B, 10-12 yr buildout, ~1.8 mi). Legacy-name filing; in nobody's pipeline count.</t>
+          <t>AUDIT WATCH: 380-ac, 3,500-home master plan approved 2024 between Maple Grove &amp; Cole at the New York Canal; apartments in later phases (15-20 yr buildout) — long-dated only.</t>
         </is>
       </c>
       <c r="H48" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2025/10/22/large-urban-project-gets-green-light-from-meridian-city-council/</t>
+          <t>https://www.ktvb.com/article/news/local/idaho-press/city-council-approves-murio-farms-3500-homes-southwest-boise/277-eb746dad-15bb-4c8e-868d-ca9d6c1e355e</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="37" t="inlineStr">
         <is>
-          <t>The District at Ten Mile (BVA + CenterCal principals)</t>
+          <t>Pine 43 VI residential (same MDA as the 270u CUP)</t>
         </is>
       </c>
       <c r="C49" s="77" t="n">
-        <v>1800</v>
+        <v>604</v>
       </c>
       <c r="D49" s="77" t="n"/>
       <c r="E49" s="37" t="n"/>
       <c r="F49" s="37" t="n"/>
       <c r="G49" s="37" t="inlineStr">
         <is>
-          <t>AUG 2026 AUDIT: 222-ac master plan NW quadrant I-84 &amp; Ten Mile broke ground May 2026 (Target, Life Time, hotels); ~1,800 residential units incl. up to 400 TH with vertical from ~June 2026. Rental MF phases unbranded/uncounted in any feed (~3.3 mi).</t>
+          <t>AUG 2026 AUDIT: H-2024-0071 (approved 10/21/2025) also allows up to 604 vertically-integrated units over ground-floor commercial (87-ft height exception) + 30 TH — up to 904 total units in the Pine 43 revamp (~$1B, 10-12 yr buildout, ~1.8 mi). Legacy-name filing; in nobody's pipeline count.</t>
         </is>
       </c>
       <c r="H49" s="37" t="inlineStr">
         <is>
-          <t>https://idahobusinessreview.com/2026/06/22/district-at-ten-mile-meridian-development/</t>
+          <t>https://boisedev.com/news/2025/10/22/large-urban-project-gets-green-light-from-meridian-city-council/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="37" t="inlineStr">
         <is>
-          <t>Modern Craftsman Franklin (Baron BTR, Franklin &amp; Black Cat)</t>
+          <t>The District at Ten Mile (BVA + CenterCal principals)</t>
         </is>
       </c>
       <c r="C50" s="77" t="n">
-        <v>122</v>
+        <v>1800</v>
       </c>
       <c r="D50" s="77" t="n"/>
       <c r="E50" s="37" t="n"/>
       <c r="F50" s="37" t="n"/>
       <c r="G50" s="37" t="inlineStr">
         <is>
-          <t>AUG 2026 AUDIT: 122 BTR dwellings (SFR/duplex/6-plex) filed 2023 (annexation+CUP+plat); post-2023 status UNVERIFIED — name collides with built Modern Craftsman Ten Mile. Verify with Meridian planning before counting (~4.0 mi).</t>
+          <t>AUG 2026 AUDIT: 222-ac master plan NW quadrant I-84 &amp; Ten Mile broke ground May 2026 (Target, Life Time, hotels); ~1,800 residential units incl. up to 400 TH with vertical from ~June 2026. Rental MF phases unbranded/uncounted in any feed (~3.3 mi).</t>
         </is>
       </c>
       <c r="H50" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2023/02/17/modern-craftsman-subdivision/</t>
+          <t>https://idahobusinessreview.com/2026/06/22/district-at-ten-mile-meridian-development/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="37" t="inlineStr">
         <is>
-          <t>Kleiner Trust field (Fairview &amp; Eagle, 71.8 ac C-G)</t>
-        </is>
-      </c>
-      <c r="C51" s="77" t="n"/>
+          <t>Modern Craftsman Franklin (Baron BTR, Franklin &amp; Black Cat)</t>
+        </is>
+      </c>
+      <c r="C51" s="77" t="n">
+        <v>122</v>
+      </c>
       <c r="D51" s="77" t="n"/>
       <c r="E51" s="37" t="n"/>
       <c r="F51" s="37" t="n"/>
       <c r="G51" s="37" t="inlineStr">
         <is>
-          <t>AUG 2026 AUDIT: Two ag-exempt parcels (3000 E Fairview 36.6 ac + N Eagle Rd 35.2 ac) = the ~72.5-ac Julius Kleiner family trust field. No applications, not listed, held for decades; CenterCal dropped 549 apartments at the adjacent Village expansion for lack of demand. Biggest long-term optionality in the ring; zero current motion (~2.0-2.3 mi).</t>
+          <t>AUG 2026 AUDIT: 122 BTR dwellings (SFR/duplex/6-plex) filed 2023 (annexation+CUP+plat); post-2023 status UNVERIFIED — name collides with built Modern Craftsman Ten Mile. Verify with Meridian planning before counting (~4.0 mi).</t>
         </is>
       </c>
       <c r="H51" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2022/09/20/kleiner-eagle-fairview/</t>
+          <t>https://boisedev.com/news/2023/02/17/modern-craftsman-subdivision/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="37" t="inlineStr">
         <is>
-          <t>1780 E Overland Rd (5.4 ac ag-exempt C-G)</t>
+          <t>Kleiner Trust field (Fairview &amp; Eagle, 71.8 ac C-G)</t>
         </is>
       </c>
       <c r="C52" s="77" t="n"/>
@@ -9005,15 +9159,19 @@
       <c r="F52" s="37" t="n"/>
       <c r="G52" s="37" t="inlineStr">
         <is>
-          <t>AUG 2026 AUDIT: Idle freeway-visible C-G 0.6 mi W of subject; no application, no listing, owner unverified. On a corridor where C-G→MF CUPs keep passing (Rolling Hill 200u approved 5/19/26). Nearest genuinely convertible dirt after the WinCo denial.</t>
-        </is>
-      </c>
-      <c r="H52" s="37" t="inlineStr"/>
+          <t>AUG 2026 AUDIT: Two ag-exempt parcels (3000 E Fairview 36.6 ac + N Eagle Rd 35.2 ac) = the ~72.5-ac Julius Kleiner family trust field. No applications, not listed, held for decades; CenterCal dropped 549 apartments at the adjacent Village expansion for lack of demand. Biggest long-term optionality in the ring; zero current motion (~2.0-2.3 mi).</t>
+        </is>
+      </c>
+      <c r="H52" s="37" t="inlineStr">
+        <is>
+          <t>https://boisedev.com/news/2022/09/20/kleiner-eagle-fairview/</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="B53" s="37" t="inlineStr">
         <is>
-          <t>1450 E Franklin Rd (12.8 ac ag-exempt C-G)</t>
+          <t>1780 E Overland Rd (5.4 ac ag-exempt C-G)</t>
         </is>
       </c>
       <c r="C53" s="77" t="n"/>
@@ -9022,7 +9180,7 @@
       <c r="F53" s="37" t="n"/>
       <c r="G53" s="37" t="inlineStr">
         <is>
-          <t>AUG 2026 AUDIT: Was on LoopNet ("Northeast Meridian Land"), now delisted; no application (1.2 mi). Stalled 36u OZ project across the street signals weak small-MF economics.</t>
+          <t>AUG 2026 AUDIT: Idle freeway-visible C-G 0.6 mi W of subject; no application, no listing, owner unverified. On a corridor where C-G→MF CUPs keep passing (Rolling Hill 200u approved 5/19/26). Nearest genuinely convertible dirt after the WinCo denial.</t>
         </is>
       </c>
       <c r="H53" s="37" t="inlineStr"/>
@@ -9030,7 +9188,7 @@
     <row r="54">
       <c r="B54" s="37" t="inlineStr">
         <is>
-          <t>Latitude Forty Three (675/715/955 S Wells St — benign marker)</t>
+          <t>1450 E Franklin Rd (12.8 ac ag-exempt C-G)</t>
         </is>
       </c>
       <c r="C54" s="77" t="n"/>
@@ -9039,10 +9197,27 @@
       <c r="F54" s="37" t="n"/>
       <c r="G54" s="37" t="inlineStr">
         <is>
+          <t>AUG 2026 AUDIT: Was on LoopNet ("Northeast Meridian Land"), now delisted; no application (1.2 mi). Stalled 36u OZ project across the street signals weak small-MF economics.</t>
+        </is>
+      </c>
+      <c r="H54" s="37" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="B55" s="37" t="inlineStr">
+        <is>
+          <t>Latitude Forty Three (675/715/955 S Wells St — benign marker)</t>
+        </is>
+      </c>
+      <c r="C55" s="77" t="n"/>
+      <c r="D55" s="77" t="n"/>
+      <c r="E55" s="37" t="n"/>
+      <c r="F55" s="37" t="n"/>
+      <c r="G55" s="37" t="inlineStr">
+        <is>
           <t>AUG 2026 AUDIT: H-2024-0059: 79 detached FOR-SALE homes + 1 C-N pad on the Magic View enclave 0.3 mi N. P&amp;Z rec. approval 6-0 (4/3/25); council continued repeatedly pending ITD TIA (latest 4/7/26). NOT multifamily — extinguishes the enclave's prior senior/MF potential. Logged so the closest-in application is on the map.</t>
         </is>
       </c>
-      <c r="H54" s="37" t="inlineStr"/>
+      <c r="H55" s="37" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
28-agent sweep results: 552 vacant-site verdicts + shot-down MF register
- vacant_sites_verdicts.json: 10 High / 40 Medium / 88 Low-Watch / 414 benign;
  curated per synthesis conflicts (ex-Cobalt Point, Pine 43 overlap)
- graveyard_register.md: 15 killed projects 2015-2026 with pattern read
- Land Use Analysis xlsx: new 'All Vacant Verdicts' sheet (552 rows, color-keyed)
- Supply Chart Diligence: shot-down register section + Apex Zenith and
  Victory/Ten Mile watch rows
- Supply Map: 11 gray documented-dead pins + 2 new purple watch pins (76 pins)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CQcHG3mGNNEuNdk4jQMCJB
</commit_message>
<xml_diff>
--- a/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
+++ b/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
@@ -893,7 +893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:M61"/>
+  <dimension ref="B2:M61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="79" min="1" max="1"/>
@@ -3099,7 +3099,6 @@
       </c>
     </row>
     <row r="59"/>
-    <row r="60"/>
     <row r="61">
       <c r="B61" s="84" t="inlineStr">
         <is>
@@ -3127,7 +3126,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z75"/>
+  <dimension ref="B1:Z75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="1"/>
   <cols>
     <col width="2.44140625" customWidth="1" style="79" min="1" max="1"/>
@@ -7833,7 +7832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A2:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="2.44140625" customWidth="1" style="79" min="1" max="1"/>
@@ -7846,7 +7845,6 @@
     <col width="36" customWidth="1" style="79" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="86" t="inlineStr">
         <is>
@@ -8690,7 +8688,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="B32" s="37" t="inlineStr">
         <is>
@@ -9218,6 +9215,481 @@
         </is>
       </c>
       <c r="H55" s="37" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="B57" s="86" t="inlineStr">
+        <is>
+          <t>SHOT-DOWN MF REGISTER (denied / withdrawn / expired / converted — 2015-2026 sweep, Aug 14 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="44" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C58" s="44" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D58" s="44" t="n"/>
+      <c r="E58" s="44" t="inlineStr">
+        <is>
+          <t>Outcome / year</t>
+        </is>
+      </c>
+      <c r="F58" s="44" t="n"/>
+      <c r="G58" s="44" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H58" s="44" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="37" t="inlineStr">
+        <is>
+          <t>Overland &amp; Wells II / "Seasons at Meridian II" (H-2022-0030)</t>
+        </is>
+      </c>
+      <c r="C59" s="77" t="n">
+        <v>345</v>
+      </c>
+      <c r="D59" s="77" t="n"/>
+      <c r="E59" s="37" t="inlineStr">
+        <is>
+          <t>DENIED Nov 2022</t>
+        </is>
+      </c>
+      <c r="F59" s="37" t="n"/>
+      <c r="G59" s="37" t="inlineStr">
+        <is>
+          <t>Touching parcel. Employment-land loss, failing intersections, MF over-concentration. WinCo owns; retail pads marketed. ~5% revival, earliest ~2030.</t>
+        </is>
+      </c>
+      <c r="H59" s="37" t="inlineStr">
+        <is>
+          <t>meetings.municode.com MERIDIANID 11/9/2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="37" t="inlineStr">
+        <is>
+          <t>Andorra Senior Living (H-2019-0127) + 2021 assisted-living</t>
+        </is>
+      </c>
+      <c r="C60" s="77" t="n">
+        <v>164</v>
+      </c>
+      <c r="D60" s="77" t="n"/>
+      <c r="E60" s="37" t="inlineStr">
+        <is>
+          <t>EXPIRED 2020 / DENIED 2021</t>
+        </is>
+      </c>
+      <c r="F60" s="37" t="n"/>
+      <c r="G60" s="37" t="inlineStr">
+        <is>
+          <t>Magic View enclave 0.3 mi: senior annexation approved 2019 but DA never signed; 2021 assisted-living denied. Site now in the for-sale Latitude 43 plat.</t>
+        </is>
+      </c>
+      <c r="H60" s="37" t="inlineStr">
+        <is>
+          <t>Meridian records</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="37" t="inlineStr">
+        <is>
+          <t>Cobalt Point (H-2022-0042)</t>
+        </is>
+      </c>
+      <c r="C61" s="77" t="n">
+        <v>264</v>
+      </c>
+      <c r="D61" s="77" t="n"/>
+      <c r="E61" s="37" t="inlineStr">
+        <is>
+          <t>WITHDRAWN Dec 2022</t>
+        </is>
+      </c>
+      <c r="F61" s="37" t="n"/>
+      <c r="G61" s="37" t="inlineStr">
+        <is>
+          <t>11.95-ac C-G at Copper Point/Cobalt Point Way (0.8 mi); never re-filed; land still vacant — entitled-once dirt, kept Low-Watch.</t>
+        </is>
+      </c>
+      <c r="H61" s="37" t="inlineStr">
+        <is>
+          <t>Meridian records</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="37" t="inlineStr">
+        <is>
+          <t>Fairview Apartments (H-2023-0001)</t>
+        </is>
+      </c>
+      <c r="C62" s="77" t="n">
+        <v>150</v>
+      </c>
+      <c r="D62" s="77" t="n"/>
+      <c r="E62" s="37" t="inlineStr">
+        <is>
+          <t>WITHDRAWN Jun 2023</t>
+        </is>
+      </c>
+      <c r="F62" s="37" t="n"/>
+      <c r="G62" s="37" t="inlineStr">
+        <is>
+          <t>1005 E Fairview; site re-tenanted as RV dealership Apr 2024.</t>
+        </is>
+      </c>
+      <c r="H62" s="37" t="inlineStr">
+        <is>
+          <t>Meridian records</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="37" t="inlineStr">
+        <is>
+          <t>The 10 at Meridian (Elk Ventures)</t>
+        </is>
+      </c>
+      <c r="C63" s="77" t="n">
+        <v>559</v>
+      </c>
+      <c r="D63" s="77" t="n"/>
+      <c r="E63" s="37" t="inlineStr">
+        <is>
+          <t>ABANDONED ~2024</t>
+        </is>
+      </c>
+      <c r="F63" s="37" t="n"/>
+      <c r="G63" s="37" t="inlineStr">
+        <is>
+          <t>SW Franklin &amp; Ten Mile; superseded by Gateway (#39) / Outer Banks (#33) — VERIFY footprint split.</t>
+        </is>
+      </c>
+      <c r="H63" s="37" t="inlineStr">
+        <is>
+          <t>BoiseDev</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="37" t="inlineStr">
+        <is>
+          <t>Rolling Hill original plan</t>
+        </is>
+      </c>
+      <c r="C64" s="77" t="n">
+        <v>154</v>
+      </c>
+      <c r="D64" s="77" t="n"/>
+      <c r="E64" s="37" t="inlineStr">
+        <is>
+          <t>DENIED 2024</t>
+        </is>
+      </c>
+      <c r="F64" s="37" t="n"/>
+      <c r="G64" s="37" t="inlineStr">
+        <is>
+          <t>First Assemble plan denied (county enclave); revised 200u APPROVED 5/19/2026 → row #37.</t>
+        </is>
+      </c>
+      <c r="H64" s="37" t="inlineStr">
+        <is>
+          <t>BoiseDev 5/20/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="37" t="inlineStr">
+        <is>
+          <t>Madison Town Square</t>
+        </is>
+      </c>
+      <c r="C65" s="77" t="n">
+        <v>251</v>
+      </c>
+      <c r="D65" s="77" t="n"/>
+      <c r="E65" s="37" t="inlineStr">
+        <is>
+          <t>WITHDRAWN Jun 2024</t>
+        </is>
+      </c>
+      <c r="F65" s="37" t="n"/>
+      <c r="G65" s="37" t="inlineStr">
+        <is>
+          <t>Old Sears site, 460 N Milwaukee (Boise); pulled; site for sale.</t>
+        </is>
+      </c>
+      <c r="H65" s="37" t="inlineStr">
+        <is>
+          <t>BoiseDev</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="37" t="inlineStr">
+        <is>
+          <t>The Bridge at Village at Meridian</t>
+        </is>
+      </c>
+      <c r="C66" s="77" t="n">
+        <v>549</v>
+      </c>
+      <c r="D66" s="77" t="n"/>
+      <c r="E66" s="37" t="inlineStr">
+        <is>
+          <t>ABANDONED Aug 2024</t>
+        </is>
+      </c>
+      <c r="F66" s="37" t="n"/>
+      <c r="G66" s="37" t="inlineStr">
+        <is>
+          <t>CenterCal dropped residential expansion "for lack of demand"; retail-only rebuild.</t>
+        </is>
+      </c>
+      <c r="H66" s="37" t="inlineStr">
+        <is>
+          <t>BoiseDev 8/19/24</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="37" t="inlineStr">
+        <is>
+          <t>Lake Hazel &amp; Five Mile (Ada County)</t>
+        </is>
+      </c>
+      <c r="C67" s="77" t="n">
+        <v>128</v>
+      </c>
+      <c r="D67" s="77" t="n"/>
+      <c r="E67" s="37" t="inlineStr">
+        <is>
+          <t>DENIED 2022 &amp; 2024</t>
+        </is>
+      </c>
+      <c r="F67" s="37" t="n"/>
+      <c r="G67" s="37" t="inlineStr">
+        <is>
+          <t>128u then 118u denied; 2025 commercial-only approved. Dead as MF.</t>
+        </is>
+      </c>
+      <c r="H67" s="37" t="inlineStr">
+        <is>
+          <t>Ada County records</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="37" t="inlineStr">
+        <is>
+          <t>Centrepoint — Devco affordable (H-2024-0019)</t>
+        </is>
+      </c>
+      <c r="C68" s="77" t="n">
+        <v>239</v>
+      </c>
+      <c r="D68" s="77" t="n"/>
+      <c r="E68" s="37" t="inlineStr">
+        <is>
+          <t>WITHDRAWN 2025</t>
+        </is>
+      </c>
+      <c r="F68" s="37" t="n"/>
+      <c r="G68" s="37" t="inlineStr">
+        <is>
+          <t>Affordable plan killed; superseded by 213u market-rate approval Dec 2025 → row #32.</t>
+        </is>
+      </c>
+      <c r="H68" s="37" t="inlineStr">
+        <is>
+          <t>Meridian records</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="37" t="inlineStr">
+        <is>
+          <t>Newkirk (H-2024-0043)</t>
+        </is>
+      </c>
+      <c r="C69" s="77" t="n">
+        <v>216</v>
+      </c>
+      <c r="D69" s="77" t="n"/>
+      <c r="E69" s="37" t="inlineStr">
+        <is>
+          <t>CONVERTED Feb 2025</t>
+        </is>
+      </c>
+      <c r="F69" s="37" t="n"/>
+      <c r="G69" s="37" t="inlineStr">
+        <is>
+          <t>Approved 216 apartments converted to 95 for-sale attached homes (Franklin &amp; Black Cat).</t>
+        </is>
+      </c>
+      <c r="H69" s="37" t="inlineStr">
+        <is>
+          <t>BoiseDev 2/13/25</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="37" t="inlineStr">
+        <is>
+          <t>The Hummingbird</t>
+        </is>
+      </c>
+      <c r="C70" s="77" t="n">
+        <v>170</v>
+      </c>
+      <c r="D70" s="77" t="n"/>
+      <c r="E70" s="37" t="inlineStr">
+        <is>
+          <t>EXPIRED spring 2025</t>
+        </is>
+      </c>
+      <c r="F70" s="37" t="n"/>
+      <c r="G70" s="37" t="inlineStr">
+        <is>
+          <t>60 N Cole Rd; approval lapsed; aquarium expansion planned instead.</t>
+        </is>
+      </c>
+      <c r="H70" s="37" t="inlineStr">
+        <is>
+          <t>BoiseDev 8/18/25</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="37" t="inlineStr">
+        <is>
+          <t>Union 93</t>
+        </is>
+      </c>
+      <c r="C71" s="77" t="n">
+        <v>93</v>
+      </c>
+      <c r="D71" s="77" t="n"/>
+      <c r="E71" s="37" t="inlineStr">
+        <is>
+          <t>FORECLOSED Oct 2025</t>
+        </is>
+      </c>
+      <c r="F71" s="37" t="n"/>
+      <c r="G71" s="37" t="inlineStr">
+        <is>
+          <t>Main &amp; Broadway skeleton foreclosed/auctioned; superseded by Heritage Square 250u → row #35.</t>
+        </is>
+      </c>
+      <c r="H71" s="37" t="inlineStr">
+        <is>
+          <t>BoiseDev</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="37" t="inlineStr">
+        <is>
+          <t>Tanner Creek original (Schulz)</t>
+        </is>
+      </c>
+      <c r="C72" s="77" t="n">
+        <v>272</v>
+      </c>
+      <c r="D72" s="77" t="n"/>
+      <c r="E72" s="37" t="inlineStr">
+        <is>
+          <t>DENIED 2018</t>
+        </is>
+      </c>
+      <c r="F72" s="37" t="n"/>
+      <c r="G72" s="37" t="inlineStr">
+        <is>
+          <t>Waltman Ln; corridor later approved as phased Tanner Creek (280 apts, CBH) — on watch list.</t>
+        </is>
+      </c>
+      <c r="H72" s="37" t="inlineStr">
+        <is>
+          <t>Meridian records</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>(pattern read)</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Council kills big MF at retail/employment nodes (protective for subject); denial is often round one — Rolling Hill/Centrepoint/Union 93/Tanner Creek all returned in new form; Magic View enclave killed senior/MF 3x; ~2,100 units died in-ring 2024-2025. Dormant-but-entitled deals (Records #38, Victory Flats #41, Ascent #46, 12548 #45, OZ #47) remain in the chart, NOT here. Syringa #40 is contested-live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="86" t="inlineStr">
+        <is>
+          <t>SHADOW WATCH — ADDED AUG 14 2026 (agent sweep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="37" t="inlineStr">
+        <is>
+          <t>Apex Zenith (Brighton) — Lake Hazel &amp; Meridian Rd</t>
+        </is>
+      </c>
+      <c r="C76" s="77" t="n"/>
+      <c r="D76" s="77" t="n"/>
+      <c r="E76" s="37" t="n"/>
+      <c r="F76" s="37" t="n"/>
+      <c r="G76" s="37" t="inlineStr">
+        <is>
+          <t>AUG 2026 SWEEP: Annexation/rezone/DA approved 4-1 Jan 2025; application references MF units; Costco portion under construction (Aug 2026 opening target). Southern ring edge (~4 mi); MF phases undated.</t>
+        </is>
+      </c>
+      <c r="H76" s="37" t="inlineStr">
+        <is>
+          <t>BoiseDev / Meridian records</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="37" t="inlineStr">
+        <is>
+          <t>Victory &amp; Ten Mile mixed-use pre-app (~142 ac)</t>
+        </is>
+      </c>
+      <c r="C77" s="77" t="n"/>
+      <c r="D77" s="77" t="n"/>
+      <c r="E77" s="37" t="n"/>
+      <c r="F77" s="37" t="n"/>
+      <c r="G77" s="37" t="inlineStr">
+        <is>
+          <t>AUG 2026 SWEEP: Oct 2025 pre-application concept (Mark Bottles RE / West Ada SD land) with a second housing product plausibly attached/MF; no formal file yet (~2.9 mi).</t>
+        </is>
+      </c>
+      <c r="H77" s="37" t="inlineStr">
+        <is>
+          <t>Oct 2025 reporting</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Fix #43 Pine 43 MF: disambiguate from built Dovetail, move pin off Dovetail parcel
The 'Pine & Webb' label + address-based pin placement put row #43 on Dovetail's
parcel (1350 N Webb Way). The 270u CUP (H-2024-0071, approved 10/21/2025) is a
distinct future project in the Pine 43 expansion; renamed row, pin moved to the
expansion annexation parcel with approx caveat, Dovetail cross-noted.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CQcHG3mGNNEuNdk4jQMCJB
</commit_message>
<xml_diff>
--- a/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
+++ b/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
@@ -1638,7 +1638,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>Units: CoStar 240 vs RealPage 480; Year built: 2020/2023; Occ: CoStar 96% vs RealPage 99%</t>
+          <t>Units: CoStar 240 vs RealPage 480; Year built: 2020/2023; Occ: CoStar 96% vs RealPage 99%; inside Pine 43 master plan — distinct from proposed 270u CUP (#43)</t>
         </is>
       </c>
       <c r="M20">
@@ -1952,6 +1952,7 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="B29" s="9" t="n"/>
       <c r="C29" s="85" t="inlineStr">
@@ -2878,7 +2879,7 @@
       </c>
       <c r="C54" s="25" t="inlineStr">
         <is>
-          <t>Pine 43 Multifamily (Pine &amp; Webb)</t>
+          <t>Pine 43 Multifamily (H-2024-0071 CUP)</t>
         </is>
       </c>
       <c r="D54" s="26" t="n">
@@ -2906,7 +2907,7 @@
       <c r="J54" s="24" t="n"/>
       <c r="K54" s="25" t="inlineStr">
         <is>
-          <t>Analyst-sourced deal (not in CoStar/RealPage); Diligence: proposed</t>
+          <t>Analyst-sourced; Diligence: proposed. 270u CUP (two bldgs, 6.28 ac C-G, height exception) in the Pine 43 expansion approved 10/21/2025, E Pine Ave betw Locust Grove &amp; Hickory. DISTINCT from built Dovetail (#15, 1350 N Webb Way) in the same master plan; same MDA also allows up to 604 VI units (shadow row).</t>
         </is>
       </c>
       <c r="M54">
@@ -3685,7 +3686,7 @@
       </c>
       <c r="R18" s="37" t="inlineStr">
         <is>
-          <t>Pine 43 Multifamily (Pine &amp; Webb)</t>
+          <t>Pine 43 Multifamily (H-2024-0071 CUP)</t>
         </is>
       </c>
       <c r="S18" s="38" t="n">
@@ -7708,7 +7709,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Pine 43 Multifamily (Pine &amp; Webb)</t>
+          <t>Pine 43 Multifamily (H-2024-0071 CUP)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7832,7 +7833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H77"/>
+  <dimension ref="B1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="2.44140625" customWidth="1" style="79" min="1" max="1"/>
@@ -7845,6 +7846,7 @@
     <col width="36" customWidth="1" style="79" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="86" t="inlineStr">
         <is>
@@ -8563,7 +8565,7 @@
     <row r="27">
       <c r="B27" s="37" t="inlineStr">
         <is>
-          <t>Pine 43 Multifamily (Pine &amp; Webb)</t>
+          <t>Pine 43 Multifamily (H-2024-0071 CUP)</t>
         </is>
       </c>
       <c r="C27" s="77" t="inlineStr">
@@ -8688,6 +8690,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="B32" s="37" t="inlineStr">
         <is>
@@ -9216,6 +9219,7 @@
       </c>
       <c r="H55" s="37" t="inlineStr"/>
     </row>
+    <row r="56"/>
     <row r="57">
       <c r="B57" s="86" t="inlineStr">
         <is>
@@ -9642,6 +9646,7 @@
         </is>
       </c>
     </row>
+    <row r="74"/>
     <row r="75">
       <c r="B75" s="86" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Vanguard Village: developer identified (Endurance/Challenger = CBH org); UC status flagged for verification
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CQcHG3mGNNEuNdk4jQMCJB
</commit_message>
<xml_diff>
--- a/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
+++ b/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
@@ -1952,7 +1952,6 @@
         <v/>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="B29" s="9" t="n"/>
       <c r="C29" s="85" t="inlineStr">
@@ -2354,7 +2353,7 @@
       </c>
       <c r="H40" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Endurance Holdings / Challenger Development (CBH)</t>
         </is>
       </c>
       <c r="I40" s="22" t="n">
@@ -2365,7 +2364,11 @@
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K40" s="18" t="n"/>
+      <c r="K40" s="18" t="inlineStr">
+        <is>
+          <t>Developer: Endurance Holdings LLC + Challenger Development Inc (Corey Barton/CBH org). Evolved from 2022 "Vanguard Commons" 432u filing. UC per CoStar (=its entire 5-mi UC series, 552u) but NO C-MULTI permit found in Meridian public reports 2025-26 — VERIFY construction status before relying on Q1 2028 delivery.</t>
+        </is>
+      </c>
       <c r="M40">
         <f>IFERROR(VALUE(RIGHT(E40,4))*4+MATCH(LEFT(E40,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
@@ -2417,6 +2420,7 @@
         <v/>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="B43" s="23" t="n"/>
       <c r="C43" s="83" t="inlineStr">
@@ -7066,6 +7070,11 @@
           <t>CoStar</t>
         </is>
       </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Aug 2026: developer = Endurance Holdings/Challenger (CBH); ex-Vanguard Commons 432u (2022); CoStar UC flag unconfirmed by city permit record — verify</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7833,7 +7842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H77"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="2.44140625" customWidth="1" style="79" min="1" max="1"/>
@@ -8763,83 +8772,89 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="86" t="inlineStr">
+      <c r="B35" s="37" t="inlineStr">
+        <is>
+          <t>Vanguard Village</t>
+        </is>
+      </c>
+      <c r="C35" s="77" t="n">
+        <v>552</v>
+      </c>
+      <c r="D35" s="77" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E35" s="37" t="inlineStr">
+        <is>
+          <t>under construction per CoStar - VERIFY (no city permit found)</t>
+        </is>
+      </c>
+      <c r="F35" s="37" t="n"/>
+      <c r="G35" s="37" t="inlineStr">
+        <is>
+          <t>AUG 2026: Developer identified = Endurance Holdings LLC + Challenger Development Inc (Corey Barton / CBH Homes org; same family as Yellowstone #16). Filed 2022 as "Vanguard Commons" (432u: 3-story apts + 2-story TH, 760-1,690 SF); DA amendment hearings into Sept 2024; CoStar now carries 552u UC / Q1 2028 — and its whole 5-mi UC series equals this one deal (552u), implying observed construction. BUT no C-MULTI permit for 1085 S Ten Mile appears in Meridian public permit reports 2025-26 (only unrelated commercial on Vanguard Way) and no groundbreaking press. Verify with Meridian Building or site visit before relying on delivery timing.</t>
+        </is>
+      </c>
+      <c r="H35" s="37" t="inlineStr">
+        <is>
+          <t>https://boisedev.com/news/2022/08/01/vanguard-commons-meridian/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="86" t="inlineStr">
         <is>
           <t>SHADOW SUPPLY (latent / untracked — watch list)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="B36" s="44" t="inlineStr">
+    <row r="37">
+      <c r="B37" s="44" t="inlineStr">
         <is>
           <t>Property / Site</t>
         </is>
       </c>
-      <c r="C36" s="44" t="inlineStr">
+      <c r="C37" s="44" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="D36" s="44" t="inlineStr">
+      <c r="D37" s="44" t="inlineStr">
         <is>
           <t>Est. Delivery</t>
         </is>
       </c>
-      <c r="E36" s="44" t="inlineStr">
+      <c r="E37" s="44" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F36" s="44" t="inlineStr">
+      <c r="F37" s="44" t="inlineStr">
         <is>
           <t>Leasing Pace</t>
         </is>
       </c>
-      <c r="G36" s="44" t="inlineStr">
+      <c r="G37" s="44" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H36" s="44" t="inlineStr">
+      <c r="H37" s="44" t="inlineStr">
         <is>
           <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="37" t="inlineStr">
-        <is>
-          <t>Emblem Meridian (Quarterra) / Artisan Victory Market site</t>
-        </is>
-      </c>
-      <c r="C37" s="77" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
-      </c>
-      <c r="D37" s="77" t="n"/>
-      <c r="E37" s="37" t="n"/>
-      <c r="F37" s="37" t="n"/>
-      <c r="G37" s="37" t="inlineStr">
-        <is>
-          <t>PROMOTED Aug 2026 to pipeline row #44 (250u) — kept here for history. Land-use analysis site SM-76: ~12-ac BPS Eagle Road LLC assemblage on S Eagle Rd. 'Artisan Victory Market' (H-2022-0066) approved 2023 for 131 build-to-rent units + commercial but never built; superseded by Quarterra's 'Emblem Meridian' ~250-unit concept (pre-application June 2026). Closest large latent MF site to the subject (~1 mi). | AUG 2026 AUDIT: formal early plans FILED June 2026 — 250 units (apts+TH) on ~13 ac (BoiseDev 6/10/26). Nearest live MF application to the subject (1.0 mi).</t>
-        </is>
-      </c>
-      <c r="H37" s="37" t="inlineStr">
-        <is>
-          <t>https://boisedev.com/news/2026/06/10/meridian-emblem-victory-eagle-homes-apartment/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="37" t="inlineStr">
         <is>
-          <t>Tanner Creek apartments (Waltman/Johnson Ln)</t>
+          <t>Emblem Meridian (Quarterra) / Artisan Victory Market site</t>
         </is>
       </c>
       <c r="C38" s="77" t="inlineStr">
         <is>
-          <t>280</t>
+          <t>250</t>
         </is>
       </c>
       <c r="D38" s="77" t="n"/>
@@ -8847,24 +8862,24 @@
       <c r="F38" s="37" t="n"/>
       <c r="G38" s="37" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-15: Tanner Creek (heard Nov 2023; moved forward) — 83 SF homes + 45 townhomes + 280 phased apartments on ~38 ac, paired with ~30-ac Hawkins commercial between I-84 and Waltman Ln. Residential now being built by CBH Homes; the 280-unit apartment component is latent supply not yet in the CoStar/RealPage pipeline.</t>
+          <t>PROMOTED Aug 2026 to pipeline row #44 (250u) — kept here for history. Land-use analysis site SM-76: ~12-ac BPS Eagle Road LLC assemblage on S Eagle Rd. 'Artisan Victory Market' (H-2022-0066) approved 2023 for 131 build-to-rent units + commercial but never built; superseded by Quarterra's 'Emblem Meridian' ~250-unit concept (pre-application June 2026). Closest large latent MF site to the subject (~1 mi). | AUG 2026 AUDIT: formal early plans FILED June 2026 — 250 units (apts+TH) on ~13 ac (BoiseDev 6/10/26). Nearest live MF application to the subject (1.0 mi).</t>
         </is>
       </c>
       <c r="H38" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2023/11/28/plans-for-two-large-developments-off-i-84-and-meridian-rd-move-forward/</t>
+          <t>https://boisedev.com/news/2026/06/10/meridian-emblem-victory-eagle-homes-apartment/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="37" t="inlineStr">
         <is>
-          <t>Graycliff Estates R-40 block</t>
+          <t>Tanner Creek apartments (Waltman/Johnson Ln)</t>
         </is>
       </c>
       <c r="C39" s="77" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>280</t>
         </is>
       </c>
       <c r="D39" s="77" t="n"/>
@@ -8872,40 +8887,44 @@
       <c r="F39" s="37" t="n"/>
       <c r="G39" s="37" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-3: Graycliff Estates (Star Development) approved preliminary plat of ~200 SF homes PLUS 224 apartments (R-40 high-density block) on ~52 ac; SF portion building since 2021. The 224-unit apartment block remains unbuilt latent supply. | AUG 2026 AUDIT: confirmed still unbuilt; no 2026 hearing/permit activity found.</t>
+          <t>Land-use analysis site SM-15: Tanner Creek (heard Nov 2023; moved forward) — 83 SF homes + 45 townhomes + 280 phased apartments on ~38 ac, paired with ~30-ac Hawkins commercial between I-84 and Waltman Ln. Residential now being built by CBH Homes; the 280-unit apartment component is latent supply not yet in the CoStar/RealPage pipeline.</t>
         </is>
       </c>
       <c r="H39" s="37" t="inlineStr">
         <is>
-          <t>https://www.weknowboise.com/graycliff-estates.php</t>
+          <t>https://boisedev.com/news/2023/11/28/plans-for-two-large-developments-off-i-84-and-meridian-rd-move-forward/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="37" t="inlineStr">
         <is>
-          <t>Touchmark Meadow Lake Village expansion</t>
-        </is>
-      </c>
-      <c r="C40" s="77" t="n"/>
+          <t>Graycliff Estates R-40 block</t>
+        </is>
+      </c>
+      <c r="C40" s="77" t="inlineStr">
+        <is>
+          <t>224</t>
+        </is>
+      </c>
       <c r="D40" s="77" t="n"/>
       <c r="E40" s="37" t="n"/>
       <c r="F40" s="37" t="n"/>
       <c r="G40" s="37" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-9: ~64 undeveloped ac of Touchmark's ~121-ac senior community. July 2025 development-modification agreement + rezone + PUD in progress to a broader 'Touchmark Mixed Use' (mixed housing types). Senior-oriented, but adds rental housing capacity 1.5 mi from subject.</t>
+          <t>Land-use analysis site SM-3: Graycliff Estates (Star Development) approved preliminary plat of ~200 SF homes PLUS 224 apartments (R-40 high-density block) on ~52 ac; SF portion building since 2021. The 224-unit apartment block remains unbuilt latent supply. | AUG 2026 AUDIT: confirmed still unbuilt; no 2026 hearing/permit activity found.</t>
         </is>
       </c>
       <c r="H40" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2025/07/14/touchmark-meridian-meadowlake-mixed-use/</t>
+          <t>https://www.weknowboise.com/graycliff-estates.php</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="37" t="inlineStr">
         <is>
-          <t>Ten Mile Crossing residual HDR parcels</t>
+          <t>Touchmark Meadow Lake Village expansion</t>
         </is>
       </c>
       <c r="C41" s="77" t="n"/>
@@ -8914,19 +8933,19 @@
       <c r="F41" s="37" t="n"/>
       <c r="G41" s="37" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-4: residential portion (R-15/R-8) of Brighton's Ten Mile Crossing at SW Overland &amp; Ten Mile — partially built (Cortland South Meridian + CBH SF); remaining High-Density Residential parcels planned/dormant, including an 8.6-ac and a 14.4-ac R-15 vacant parcel (highest-interest sites in the land-use ranking). Note: South Ridge II (164u UC, tracked in the chart) is rising in this same corridor.</t>
+          <t>Land-use analysis site SM-9: ~64 undeveloped ac of Touchmark's ~121-ac senior community. July 2025 development-modification agreement + rezone + PUD in progress to a broader 'Touchmark Mixed Use' (mixed housing types). Senior-oriented, but adds rental housing capacity 1.5 mi from subject.</t>
         </is>
       </c>
       <c r="H41" s="37" t="inlineStr">
         <is>
-          <t>https://www.brighton.co/brighton-place/ten-mile-crossing/</t>
+          <t>https://boisedev.com/news/2025/07/14/touchmark-meridian-meadowlake-mixed-use/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="37" t="inlineStr">
         <is>
-          <t>Brighton Apex R-15 parcel (Lake Hazel)</t>
+          <t>Ten Mile Crossing residual HDR parcels</t>
         </is>
       </c>
       <c r="C42" s="77" t="n"/>
@@ -8935,19 +8954,19 @@
       <c r="F42" s="37" t="n"/>
       <c r="G42" s="37" t="inlineStr">
         <is>
-          <t>Land-use analysis site SM-61: 15.1-ac R-15 (med-high-density) parcel on E Lake Hazel Rd inside Brighton's approved Apex/Pinnacle master-plan footprint; adjacent phases actively building. Latent MF-capable ground in the fast-growing S Meridian corridor.</t>
+          <t>Land-use analysis site SM-4: residential portion (R-15/R-8) of Brighton's Ten Mile Crossing at SW Overland &amp; Ten Mile — partially built (Cortland South Meridian + CBH SF); remaining High-Density Residential parcels planned/dormant, including an 8.6-ac and a 14.4-ac R-15 vacant parcel (highest-interest sites in the land-use ranking). Note: South Ridge II (164u UC, tracked in the chart) is rising in this same corridor.</t>
         </is>
       </c>
       <c r="H42" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2024/12/20/brighton-pinnacle-costco-meridian/</t>
+          <t>https://www.brighton.co/brighton-place/ten-mile-crossing/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="37" t="inlineStr">
         <is>
-          <t>Outer Banks Subdivision (TM Creek / Cobalt Dr)</t>
+          <t>Brighton Apex R-15 parcel (Lake Hazel)</t>
         </is>
       </c>
       <c r="C43" s="77" t="n"/>
@@ -8956,49 +8975,45 @@
       <c r="F43" s="37" t="n"/>
       <c r="G43" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROMOTED Aug 2026 to pipeline row #33 "Outer Banks Apartments" (516u, groundbreaking expected 2026) — kept here for history. </t>
+          <t>Land-use analysis site SM-61: 15.1-ac R-15 (med-high-density) parcel on E Lake Hazel Rd inside Brighton's approved Apex/Pinnacle master-plan footprint; adjacent phases actively building. Latent MF-capable ground in the fast-growing S Meridian corridor.</t>
         </is>
       </c>
       <c r="H43" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2021/12/17/outer-banks-pera-place/</t>
+          <t>https://boisedev.com/news/2024/12/20/brighton-pinnacle-costco-meridian/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="37" t="inlineStr">
         <is>
-          <t>Grandview Communities (Lake Hazel &amp; Linder)</t>
-        </is>
-      </c>
-      <c r="C44" s="77" t="inlineStr">
-        <is>
-          <t>130</t>
-        </is>
-      </c>
+          <t>Outer Banks Subdivision (TM Creek / Cobalt Dr)</t>
+        </is>
+      </c>
+      <c r="C44" s="77" t="n"/>
       <c r="D44" s="77" t="n"/>
       <c r="E44" s="37" t="n"/>
       <c r="F44" s="37" t="n"/>
       <c r="G44" s="37" t="inlineStr">
         <is>
-          <t>AUDIT WATCH: 79-ac pre-application (July 2025) at NE corner Lake Hazel &amp; Linder — ~510 homes incl. ~130 apartments + 176 TH/cluster; no formal H-file or hearing yet; sits near the southern ring edge (~4.5 mi).</t>
+          <t xml:space="preserve">PROMOTED Aug 2026 to pipeline row #33 "Outer Banks Apartments" (516u, groundbreaking expected 2026) — kept here for history. </t>
         </is>
       </c>
       <c r="H44" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2025/07/07/hundreds-of-homes-apartments-planned-for-lake-hazel-and-linder/</t>
+          <t>https://boisedev.com/news/2021/12/17/outer-banks-pera-place/</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="37" t="inlineStr">
         <is>
-          <t>Discovery project (Lake Hazel &amp; Locust Grove)</t>
+          <t>Grandview Communities (Lake Hazel &amp; Linder)</t>
         </is>
       </c>
       <c r="C45" s="77" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>130</t>
         </is>
       </c>
       <c r="D45" s="77" t="n"/>
@@ -9006,40 +9021,44 @@
       <c r="F45" s="37" t="n"/>
       <c r="G45" s="37" t="inlineStr">
         <is>
-          <t>AUDIT WATCH: April 2024 pre-application for 200+ units (nine 3-story buildings + TH/SFR) on ~20 ac by Discovery Park; no formal application since — dormant but the land is teed up (~3.5 mi).</t>
+          <t>AUDIT WATCH: 79-ac pre-application (July 2025) at NE corner Lake Hazel &amp; Linder — ~510 homes incl. ~130 apartments + 176 TH/cluster; no formal H-file or hearing yet; sits near the southern ring edge (~4.5 mi).</t>
         </is>
       </c>
       <c r="H45" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2024/04/12/200-apartments-meridian-discovery/</t>
+          <t>https://boisedev.com/news/2025/07/07/hundreds-of-homes-apartments-planned-for-lake-hazel-and-linder/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="37" t="inlineStr">
         <is>
-          <t>709 N Cole Rd (city land trust)</t>
-        </is>
-      </c>
-      <c r="C46" s="77" t="n"/>
+          <t>Discovery project (Lake Hazel &amp; Locust Grove)</t>
+        </is>
+      </c>
+      <c r="C46" s="77" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
       <c r="D46" s="77" t="n"/>
       <c r="E46" s="37" t="n"/>
       <c r="F46" s="37" t="n"/>
       <c r="G46" s="37" t="inlineStr">
         <is>
-          <t>AUDIT WATCH: City of Boise closing (July 2026) on 1.64 ac by Boise Towne Square for future affordable housing (prior owner proposed 71 micro-units in 2021); no developer or program yet — 2029+ speculative. Same parcel as the excluded 'Cole Road' RealPage entry.</t>
+          <t>AUDIT WATCH: April 2024 pre-application for 200+ units (nine 3-story buildings + TH/SFR) on ~20 ac by Discovery Park; no formal application since — dormant but the land is teed up (~3.5 mi).</t>
         </is>
       </c>
       <c r="H46" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2026/06/01/709-cole-boise/</t>
+          <t>https://boisedev.com/news/2024/04/12/200-apartments-meridian-discovery/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="37" t="inlineStr">
         <is>
-          <t>Aren east phase (verify)</t>
+          <t>709 N Cole Rd (city land trust)</t>
         </is>
       </c>
       <c r="C47" s="77" t="n"/>
@@ -9048,19 +9067,19 @@
       <c r="F47" s="37" t="n"/>
       <c r="G47" s="37" t="inlineStr">
         <is>
-          <t>AUDIT WATCH: The Aren (396u, delivered 2024) was planned as two phases at Eagle View Landing; verify whether the east-phase (~200u) buildings are fully delivered within the tracked 396 or represent additional untracked pipeline.</t>
+          <t>AUDIT WATCH: City of Boise closing (July 2026) on 1.64 ac by Boise Towne Square for future affordable housing (prior owner proposed 71 micro-units in 2021); no developer or program yet — 2029+ speculative. Same parcel as the excluded 'Cole Road' RealPage entry.</t>
         </is>
       </c>
       <c r="H47" s="37" t="inlineStr">
         <is>
-          <t>https://arenmeridian.com/</t>
+          <t>https://boisedev.com/news/2026/06/01/709-cole-boise/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="37" t="inlineStr">
         <is>
-          <t>Murio Farms MF phases (SW Boise)</t>
+          <t>Aren east phase (verify)</t>
         </is>
       </c>
       <c r="C48" s="77" t="n"/>
@@ -9069,109 +9088,109 @@
       <c r="F48" s="37" t="n"/>
       <c r="G48" s="37" t="inlineStr">
         <is>
-          <t>AUDIT WATCH: 380-ac, 3,500-home master plan approved 2024 between Maple Grove &amp; Cole at the New York Canal; apartments in later phases (15-20 yr buildout) — long-dated only.</t>
+          <t>AUDIT WATCH: The Aren (396u, delivered 2024) was planned as two phases at Eagle View Landing; verify whether the east-phase (~200u) buildings are fully delivered within the tracked 396 or represent additional untracked pipeline.</t>
         </is>
       </c>
       <c r="H48" s="37" t="inlineStr">
         <is>
-          <t>https://www.ktvb.com/article/news/local/idaho-press/city-council-approves-murio-farms-3500-homes-southwest-boise/277-eb746dad-15bb-4c8e-868d-ca9d6c1e355e</t>
+          <t>https://arenmeridian.com/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="37" t="inlineStr">
         <is>
-          <t>Pine 43 VI residential (same MDA as the 270u CUP)</t>
-        </is>
-      </c>
-      <c r="C49" s="77" t="n">
-        <v>604</v>
-      </c>
+          <t>Murio Farms MF phases (SW Boise)</t>
+        </is>
+      </c>
+      <c r="C49" s="77" t="n"/>
       <c r="D49" s="77" t="n"/>
       <c r="E49" s="37" t="n"/>
       <c r="F49" s="37" t="n"/>
       <c r="G49" s="37" t="inlineStr">
         <is>
-          <t>AUG 2026 AUDIT: H-2024-0071 (approved 10/21/2025) also allows up to 604 vertically-integrated units over ground-floor commercial (87-ft height exception) + 30 TH — up to 904 total units in the Pine 43 revamp (~$1B, 10-12 yr buildout, ~1.8 mi). Legacy-name filing; in nobody's pipeline count.</t>
+          <t>AUDIT WATCH: 380-ac, 3,500-home master plan approved 2024 between Maple Grove &amp; Cole at the New York Canal; apartments in later phases (15-20 yr buildout) — long-dated only.</t>
         </is>
       </c>
       <c r="H49" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2025/10/22/large-urban-project-gets-green-light-from-meridian-city-council/</t>
+          <t>https://www.ktvb.com/article/news/local/idaho-press/city-council-approves-murio-farms-3500-homes-southwest-boise/277-eb746dad-15bb-4c8e-868d-ca9d6c1e355e</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="37" t="inlineStr">
         <is>
-          <t>The District at Ten Mile (BVA + CenterCal principals)</t>
+          <t>Pine 43 VI residential (same MDA as the 270u CUP)</t>
         </is>
       </c>
       <c r="C50" s="77" t="n">
-        <v>1800</v>
+        <v>604</v>
       </c>
       <c r="D50" s="77" t="n"/>
       <c r="E50" s="37" t="n"/>
       <c r="F50" s="37" t="n"/>
       <c r="G50" s="37" t="inlineStr">
         <is>
-          <t>AUG 2026 AUDIT: 222-ac master plan NW quadrant I-84 &amp; Ten Mile broke ground May 2026 (Target, Life Time, hotels); ~1,800 residential units incl. up to 400 TH with vertical from ~June 2026. Rental MF phases unbranded/uncounted in any feed (~3.3 mi).</t>
+          <t>AUG 2026 AUDIT: H-2024-0071 (approved 10/21/2025) also allows up to 604 vertically-integrated units over ground-floor commercial (87-ft height exception) + 30 TH — up to 904 total units in the Pine 43 revamp (~$1B, 10-12 yr buildout, ~1.8 mi). Legacy-name filing; in nobody's pipeline count.</t>
         </is>
       </c>
       <c r="H50" s="37" t="inlineStr">
         <is>
-          <t>https://idahobusinessreview.com/2026/06/22/district-at-ten-mile-meridian-development/</t>
+          <t>https://boisedev.com/news/2025/10/22/large-urban-project-gets-green-light-from-meridian-city-council/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="37" t="inlineStr">
         <is>
-          <t>Modern Craftsman Franklin (Baron BTR, Franklin &amp; Black Cat)</t>
+          <t>The District at Ten Mile (BVA + CenterCal principals)</t>
         </is>
       </c>
       <c r="C51" s="77" t="n">
-        <v>122</v>
+        <v>1800</v>
       </c>
       <c r="D51" s="77" t="n"/>
       <c r="E51" s="37" t="n"/>
       <c r="F51" s="37" t="n"/>
       <c r="G51" s="37" t="inlineStr">
         <is>
-          <t>AUG 2026 AUDIT: 122 BTR dwellings (SFR/duplex/6-plex) filed 2023 (annexation+CUP+plat); post-2023 status UNVERIFIED — name collides with built Modern Craftsman Ten Mile. Verify with Meridian planning before counting (~4.0 mi).</t>
+          <t>AUG 2026 AUDIT: 222-ac master plan NW quadrant I-84 &amp; Ten Mile broke ground May 2026 (Target, Life Time, hotels); ~1,800 residential units incl. up to 400 TH with vertical from ~June 2026. Rental MF phases unbranded/uncounted in any feed (~3.3 mi).</t>
         </is>
       </c>
       <c r="H51" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2023/02/17/modern-craftsman-subdivision/</t>
+          <t>https://idahobusinessreview.com/2026/06/22/district-at-ten-mile-meridian-development/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="37" t="inlineStr">
         <is>
-          <t>Kleiner Trust field (Fairview &amp; Eagle, 71.8 ac C-G)</t>
-        </is>
-      </c>
-      <c r="C52" s="77" t="n"/>
+          <t>Modern Craftsman Franklin (Baron BTR, Franklin &amp; Black Cat)</t>
+        </is>
+      </c>
+      <c r="C52" s="77" t="n">
+        <v>122</v>
+      </c>
       <c r="D52" s="77" t="n"/>
       <c r="E52" s="37" t="n"/>
       <c r="F52" s="37" t="n"/>
       <c r="G52" s="37" t="inlineStr">
         <is>
-          <t>AUG 2026 AUDIT: Two ag-exempt parcels (3000 E Fairview 36.6 ac + N Eagle Rd 35.2 ac) = the ~72.5-ac Julius Kleiner family trust field. No applications, not listed, held for decades; CenterCal dropped 549 apartments at the adjacent Village expansion for lack of demand. Biggest long-term optionality in the ring; zero current motion (~2.0-2.3 mi).</t>
+          <t>AUG 2026 AUDIT: 122 BTR dwellings (SFR/duplex/6-plex) filed 2023 (annexation+CUP+plat); post-2023 status UNVERIFIED — name collides with built Modern Craftsman Ten Mile. Verify with Meridian planning before counting (~4.0 mi).</t>
         </is>
       </c>
       <c r="H52" s="37" t="inlineStr">
         <is>
-          <t>https://boisedev.com/news/2022/09/20/kleiner-eagle-fairview/</t>
+          <t>https://boisedev.com/news/2023/02/17/modern-craftsman-subdivision/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="37" t="inlineStr">
         <is>
-          <t>1780 E Overland Rd (5.4 ac ag-exempt C-G)</t>
+          <t>Kleiner Trust field (Fairview &amp; Eagle, 71.8 ac C-G)</t>
         </is>
       </c>
       <c r="C53" s="77" t="n"/>
@@ -9180,15 +9199,19 @@
       <c r="F53" s="37" t="n"/>
       <c r="G53" s="37" t="inlineStr">
         <is>
-          <t>AUG 2026 AUDIT: Idle freeway-visible C-G 0.6 mi W of subject; no application, no listing, owner unverified. On a corridor where C-G→MF CUPs keep passing (Rolling Hill 200u approved 5/19/26). Nearest genuinely convertible dirt after the WinCo denial.</t>
-        </is>
-      </c>
-      <c r="H53" s="37" t="inlineStr"/>
+          <t>AUG 2026 AUDIT: Two ag-exempt parcels (3000 E Fairview 36.6 ac + N Eagle Rd 35.2 ac) = the ~72.5-ac Julius Kleiner family trust field. No applications, not listed, held for decades; CenterCal dropped 549 apartments at the adjacent Village expansion for lack of demand. Biggest long-term optionality in the ring; zero current motion (~2.0-2.3 mi).</t>
+        </is>
+      </c>
+      <c r="H53" s="37" t="inlineStr">
+        <is>
+          <t>https://boisedev.com/news/2022/09/20/kleiner-eagle-fairview/</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="37" t="inlineStr">
         <is>
-          <t>1450 E Franklin Rd (12.8 ac ag-exempt C-G)</t>
+          <t>1780 E Overland Rd (5.4 ac ag-exempt C-G)</t>
         </is>
       </c>
       <c r="C54" s="77" t="n"/>
@@ -9197,7 +9220,7 @@
       <c r="F54" s="37" t="n"/>
       <c r="G54" s="37" t="inlineStr">
         <is>
-          <t>AUG 2026 AUDIT: Was on LoopNet ("Northeast Meridian Land"), now delisted; no application (1.2 mi). Stalled 36u OZ project across the street signals weak small-MF economics.</t>
+          <t>AUG 2026 AUDIT: Idle freeway-visible C-G 0.6 mi W of subject; no application, no listing, owner unverified. On a corridor where C-G→MF CUPs keep passing (Rolling Hill 200u approved 5/19/26). Nearest genuinely convertible dirt after the WinCo denial.</t>
         </is>
       </c>
       <c r="H54" s="37" t="inlineStr"/>
@@ -9205,7 +9228,7 @@
     <row r="55">
       <c r="B55" s="37" t="inlineStr">
         <is>
-          <t>Latitude Forty Three (675/715/955 S Wells St — benign marker)</t>
+          <t>1450 E Franklin Rd (12.8 ac ag-exempt C-G)</t>
         </is>
       </c>
       <c r="C55" s="77" t="n"/>
@@ -9214,121 +9237,111 @@
       <c r="F55" s="37" t="n"/>
       <c r="G55" s="37" t="inlineStr">
         <is>
+          <t>AUG 2026 AUDIT: Was on LoopNet ("Northeast Meridian Land"), now delisted; no application (1.2 mi). Stalled 36u OZ project across the street signals weak small-MF economics.</t>
+        </is>
+      </c>
+      <c r="H55" s="37" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="B56" s="37" t="inlineStr">
+        <is>
+          <t>Latitude Forty Three (675/715/955 S Wells St — benign marker)</t>
+        </is>
+      </c>
+      <c r="C56" s="77" t="n"/>
+      <c r="D56" s="77" t="n"/>
+      <c r="E56" s="37" t="n"/>
+      <c r="F56" s="37" t="n"/>
+      <c r="G56" s="37" t="inlineStr">
+        <is>
           <t>AUG 2026 AUDIT: H-2024-0059: 79 detached FOR-SALE homes + 1 C-N pad on the Magic View enclave 0.3 mi N. P&amp;Z rec. approval 6-0 (4/3/25); council continued repeatedly pending ITD TIA (latest 4/7/26). NOT multifamily — extinguishes the enclave's prior senior/MF potential. Logged so the closest-in application is on the map.</t>
         </is>
       </c>
-      <c r="H55" s="37" t="inlineStr"/>
-    </row>
-    <row r="56"/>
-    <row r="57">
-      <c r="B57" s="86" t="inlineStr">
+      <c r="H56" s="37" t="inlineStr"/>
+    </row>
+    <row r="57"/>
+    <row r="58">
+      <c r="B58" s="86" t="inlineStr">
         <is>
           <t>SHOT-DOWN MF REGISTER (denied / withdrawn / expired / converted — 2015-2026 sweep, Aug 14 2026)</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="B58" s="44" t="inlineStr">
+    <row r="59">
+      <c r="B59" s="44" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="C58" s="44" t="inlineStr">
+      <c r="C59" s="44" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="D58" s="44" t="n"/>
-      <c r="E58" s="44" t="inlineStr">
+      <c r="D59" s="44" t="n"/>
+      <c r="E59" s="44" t="inlineStr">
         <is>
           <t>Outcome / year</t>
         </is>
       </c>
-      <c r="F58" s="44" t="n"/>
-      <c r="G58" s="44" t="inlineStr">
+      <c r="F59" s="44" t="n"/>
+      <c r="G59" s="44" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H58" s="44" t="inlineStr">
+      <c r="H59" s="44" t="inlineStr">
         <is>
           <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="B59" s="37" t="inlineStr">
-        <is>
-          <t>Overland &amp; Wells II / "Seasons at Meridian II" (H-2022-0030)</t>
-        </is>
-      </c>
-      <c r="C59" s="77" t="n">
-        <v>345</v>
-      </c>
-      <c r="D59" s="77" t="n"/>
-      <c r="E59" s="37" t="inlineStr">
-        <is>
-          <t>DENIED Nov 2022</t>
-        </is>
-      </c>
-      <c r="F59" s="37" t="n"/>
-      <c r="G59" s="37" t="inlineStr">
-        <is>
-          <t>Touching parcel. Employment-land loss, failing intersections, MF over-concentration. WinCo owns; retail pads marketed. ~5% revival, earliest ~2030.</t>
-        </is>
-      </c>
-      <c r="H59" s="37" t="inlineStr">
-        <is>
-          <t>meetings.municode.com MERIDIANID 11/9/2022</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="B60" s="37" t="inlineStr">
         <is>
-          <t>Andorra Senior Living (H-2019-0127) + 2021 assisted-living</t>
+          <t>Overland &amp; Wells II / "Seasons at Meridian II" (H-2022-0030)</t>
         </is>
       </c>
       <c r="C60" s="77" t="n">
-        <v>164</v>
+        <v>345</v>
       </c>
       <c r="D60" s="77" t="n"/>
       <c r="E60" s="37" t="inlineStr">
         <is>
-          <t>EXPIRED 2020 / DENIED 2021</t>
+          <t>DENIED Nov 2022</t>
         </is>
       </c>
       <c r="F60" s="37" t="n"/>
       <c r="G60" s="37" t="inlineStr">
         <is>
-          <t>Magic View enclave 0.3 mi: senior annexation approved 2019 but DA never signed; 2021 assisted-living denied. Site now in the for-sale Latitude 43 plat.</t>
+          <t>Touching parcel. Employment-land loss, failing intersections, MF over-concentration. WinCo owns; retail pads marketed. ~5% revival, earliest ~2030.</t>
         </is>
       </c>
       <c r="H60" s="37" t="inlineStr">
         <is>
-          <t>Meridian records</t>
+          <t>meetings.municode.com MERIDIANID 11/9/2022</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" s="37" t="inlineStr">
         <is>
-          <t>Cobalt Point (H-2022-0042)</t>
+          <t>Andorra Senior Living (H-2019-0127) + 2021 assisted-living</t>
         </is>
       </c>
       <c r="C61" s="77" t="n">
-        <v>264</v>
+        <v>164</v>
       </c>
       <c r="D61" s="77" t="n"/>
       <c r="E61" s="37" t="inlineStr">
         <is>
-          <t>WITHDRAWN Dec 2022</t>
+          <t>EXPIRED 2020 / DENIED 2021</t>
         </is>
       </c>
       <c r="F61" s="37" t="n"/>
       <c r="G61" s="37" t="inlineStr">
         <is>
-          <t>11.95-ac C-G at Copper Point/Cobalt Point Way (0.8 mi); never re-filed; land still vacant — entitled-once dirt, kept Low-Watch.</t>
+          <t>Magic View enclave 0.3 mi: senior annexation approved 2019 but DA never signed; 2021 assisted-living denied. Site now in the for-sale Latitude 43 plat.</t>
         </is>
       </c>
       <c r="H61" s="37" t="inlineStr">
@@ -9340,22 +9353,22 @@
     <row r="62">
       <c r="B62" s="37" t="inlineStr">
         <is>
-          <t>Fairview Apartments (H-2023-0001)</t>
+          <t>Cobalt Point (H-2022-0042)</t>
         </is>
       </c>
       <c r="C62" s="77" t="n">
-        <v>150</v>
+        <v>264</v>
       </c>
       <c r="D62" s="77" t="n"/>
       <c r="E62" s="37" t="inlineStr">
         <is>
-          <t>WITHDRAWN Jun 2023</t>
+          <t>WITHDRAWN Dec 2022</t>
         </is>
       </c>
       <c r="F62" s="37" t="n"/>
       <c r="G62" s="37" t="inlineStr">
         <is>
-          <t>1005 E Fairview; site re-tenanted as RV dealership Apr 2024.</t>
+          <t>11.95-ac C-G at Copper Point/Cobalt Point Way (0.8 mi); never re-filed; land still vacant — entitled-once dirt, kept Low-Watch.</t>
         </is>
       </c>
       <c r="H62" s="37" t="inlineStr">
@@ -9367,318 +9380,324 @@
     <row r="63">
       <c r="B63" s="37" t="inlineStr">
         <is>
-          <t>The 10 at Meridian (Elk Ventures)</t>
+          <t>Fairview Apartments (H-2023-0001)</t>
         </is>
       </c>
       <c r="C63" s="77" t="n">
-        <v>559</v>
+        <v>150</v>
       </c>
       <c r="D63" s="77" t="n"/>
       <c r="E63" s="37" t="inlineStr">
         <is>
-          <t>ABANDONED ~2024</t>
+          <t>WITHDRAWN Jun 2023</t>
         </is>
       </c>
       <c r="F63" s="37" t="n"/>
       <c r="G63" s="37" t="inlineStr">
         <is>
-          <t>SW Franklin &amp; Ten Mile; superseded by Gateway (#39) / Outer Banks (#33) — VERIFY footprint split.</t>
+          <t>1005 E Fairview; site re-tenanted as RV dealership Apr 2024.</t>
         </is>
       </c>
       <c r="H63" s="37" t="inlineStr">
         <is>
-          <t>BoiseDev</t>
+          <t>Meridian records</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="B64" s="37" t="inlineStr">
         <is>
-          <t>Rolling Hill original plan</t>
+          <t>The 10 at Meridian (Elk Ventures)</t>
         </is>
       </c>
       <c r="C64" s="77" t="n">
-        <v>154</v>
+        <v>559</v>
       </c>
       <c r="D64" s="77" t="n"/>
       <c r="E64" s="37" t="inlineStr">
         <is>
-          <t>DENIED 2024</t>
+          <t>ABANDONED ~2024</t>
         </is>
       </c>
       <c r="F64" s="37" t="n"/>
       <c r="G64" s="37" t="inlineStr">
         <is>
-          <t>First Assemble plan denied (county enclave); revised 200u APPROVED 5/19/2026 → row #37.</t>
+          <t>SW Franklin &amp; Ten Mile; superseded by Gateway (#39) / Outer Banks (#33) — VERIFY footprint split.</t>
         </is>
       </c>
       <c r="H64" s="37" t="inlineStr">
         <is>
-          <t>BoiseDev 5/20/26</t>
+          <t>BoiseDev</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="B65" s="37" t="inlineStr">
         <is>
-          <t>Madison Town Square</t>
+          <t>Rolling Hill original plan</t>
         </is>
       </c>
       <c r="C65" s="77" t="n">
-        <v>251</v>
+        <v>154</v>
       </c>
       <c r="D65" s="77" t="n"/>
       <c r="E65" s="37" t="inlineStr">
         <is>
-          <t>WITHDRAWN Jun 2024</t>
+          <t>DENIED 2024</t>
         </is>
       </c>
       <c r="F65" s="37" t="n"/>
       <c r="G65" s="37" t="inlineStr">
         <is>
-          <t>Old Sears site, 460 N Milwaukee (Boise); pulled; site for sale.</t>
+          <t>First Assemble plan denied (county enclave); revised 200u APPROVED 5/19/2026 → row #37.</t>
         </is>
       </c>
       <c r="H65" s="37" t="inlineStr">
         <is>
-          <t>BoiseDev</t>
+          <t>BoiseDev 5/20/26</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="B66" s="37" t="inlineStr">
         <is>
-          <t>The Bridge at Village at Meridian</t>
+          <t>Madison Town Square</t>
         </is>
       </c>
       <c r="C66" s="77" t="n">
-        <v>549</v>
+        <v>251</v>
       </c>
       <c r="D66" s="77" t="n"/>
       <c r="E66" s="37" t="inlineStr">
         <is>
-          <t>ABANDONED Aug 2024</t>
+          <t>WITHDRAWN Jun 2024</t>
         </is>
       </c>
       <c r="F66" s="37" t="n"/>
       <c r="G66" s="37" t="inlineStr">
         <is>
-          <t>CenterCal dropped residential expansion "for lack of demand"; retail-only rebuild.</t>
+          <t>Old Sears site, 460 N Milwaukee (Boise); pulled; site for sale.</t>
         </is>
       </c>
       <c r="H66" s="37" t="inlineStr">
         <is>
-          <t>BoiseDev 8/19/24</t>
+          <t>BoiseDev</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="B67" s="37" t="inlineStr">
         <is>
-          <t>Lake Hazel &amp; Five Mile (Ada County)</t>
+          <t>The Bridge at Village at Meridian</t>
         </is>
       </c>
       <c r="C67" s="77" t="n">
-        <v>128</v>
+        <v>549</v>
       </c>
       <c r="D67" s="77" t="n"/>
       <c r="E67" s="37" t="inlineStr">
         <is>
-          <t>DENIED 2022 &amp; 2024</t>
+          <t>ABANDONED Aug 2024</t>
         </is>
       </c>
       <c r="F67" s="37" t="n"/>
       <c r="G67" s="37" t="inlineStr">
         <is>
-          <t>128u then 118u denied; 2025 commercial-only approved. Dead as MF.</t>
+          <t>CenterCal dropped residential expansion "for lack of demand"; retail-only rebuild.</t>
         </is>
       </c>
       <c r="H67" s="37" t="inlineStr">
         <is>
-          <t>Ada County records</t>
+          <t>BoiseDev 8/19/24</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="B68" s="37" t="inlineStr">
         <is>
-          <t>Centrepoint — Devco affordable (H-2024-0019)</t>
+          <t>Lake Hazel &amp; Five Mile (Ada County)</t>
         </is>
       </c>
       <c r="C68" s="77" t="n">
-        <v>239</v>
+        <v>128</v>
       </c>
       <c r="D68" s="77" t="n"/>
       <c r="E68" s="37" t="inlineStr">
         <is>
-          <t>WITHDRAWN 2025</t>
+          <t>DENIED 2022 &amp; 2024</t>
         </is>
       </c>
       <c r="F68" s="37" t="n"/>
       <c r="G68" s="37" t="inlineStr">
         <is>
-          <t>Affordable plan killed; superseded by 213u market-rate approval Dec 2025 → row #32.</t>
+          <t>128u then 118u denied; 2025 commercial-only approved. Dead as MF.</t>
         </is>
       </c>
       <c r="H68" s="37" t="inlineStr">
         <is>
-          <t>Meridian records</t>
+          <t>Ada County records</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="B69" s="37" t="inlineStr">
         <is>
-          <t>Newkirk (H-2024-0043)</t>
+          <t>Centrepoint — Devco affordable (H-2024-0019)</t>
         </is>
       </c>
       <c r="C69" s="77" t="n">
-        <v>216</v>
+        <v>239</v>
       </c>
       <c r="D69" s="77" t="n"/>
       <c r="E69" s="37" t="inlineStr">
         <is>
-          <t>CONVERTED Feb 2025</t>
+          <t>WITHDRAWN 2025</t>
         </is>
       </c>
       <c r="F69" s="37" t="n"/>
       <c r="G69" s="37" t="inlineStr">
         <is>
-          <t>Approved 216 apartments converted to 95 for-sale attached homes (Franklin &amp; Black Cat).</t>
+          <t>Affordable plan killed; superseded by 213u market-rate approval Dec 2025 → row #32.</t>
         </is>
       </c>
       <c r="H69" s="37" t="inlineStr">
         <is>
-          <t>BoiseDev 2/13/25</t>
+          <t>Meridian records</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="B70" s="37" t="inlineStr">
         <is>
-          <t>The Hummingbird</t>
+          <t>Newkirk (H-2024-0043)</t>
         </is>
       </c>
       <c r="C70" s="77" t="n">
-        <v>170</v>
+        <v>216</v>
       </c>
       <c r="D70" s="77" t="n"/>
       <c r="E70" s="37" t="inlineStr">
         <is>
-          <t>EXPIRED spring 2025</t>
+          <t>CONVERTED Feb 2025</t>
         </is>
       </c>
       <c r="F70" s="37" t="n"/>
       <c r="G70" s="37" t="inlineStr">
         <is>
-          <t>60 N Cole Rd; approval lapsed; aquarium expansion planned instead.</t>
+          <t>Approved 216 apartments converted to 95 for-sale attached homes (Franklin &amp; Black Cat).</t>
         </is>
       </c>
       <c r="H70" s="37" t="inlineStr">
         <is>
-          <t>BoiseDev 8/18/25</t>
+          <t>BoiseDev 2/13/25</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="B71" s="37" t="inlineStr">
         <is>
-          <t>Union 93</t>
+          <t>The Hummingbird</t>
         </is>
       </c>
       <c r="C71" s="77" t="n">
-        <v>93</v>
+        <v>170</v>
       </c>
       <c r="D71" s="77" t="n"/>
       <c r="E71" s="37" t="inlineStr">
         <is>
-          <t>FORECLOSED Oct 2025</t>
+          <t>EXPIRED spring 2025</t>
         </is>
       </c>
       <c r="F71" s="37" t="n"/>
       <c r="G71" s="37" t="inlineStr">
         <is>
-          <t>Main &amp; Broadway skeleton foreclosed/auctioned; superseded by Heritage Square 250u → row #35.</t>
+          <t>60 N Cole Rd; approval lapsed; aquarium expansion planned instead.</t>
         </is>
       </c>
       <c r="H71" s="37" t="inlineStr">
         <is>
-          <t>BoiseDev</t>
+          <t>BoiseDev 8/18/25</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="B72" s="37" t="inlineStr">
         <is>
-          <t>Tanner Creek original (Schulz)</t>
+          <t>Union 93</t>
         </is>
       </c>
       <c r="C72" s="77" t="n">
-        <v>272</v>
+        <v>93</v>
       </c>
       <c r="D72" s="77" t="n"/>
       <c r="E72" s="37" t="inlineStr">
         <is>
-          <t>DENIED 2018</t>
+          <t>FORECLOSED Oct 2025</t>
         </is>
       </c>
       <c r="F72" s="37" t="n"/>
       <c r="G72" s="37" t="inlineStr">
         <is>
+          <t>Main &amp; Broadway skeleton foreclosed/auctioned; superseded by Heritage Square 250u → row #35.</t>
+        </is>
+      </c>
+      <c r="H72" s="37" t="inlineStr">
+        <is>
+          <t>BoiseDev</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="37" t="inlineStr">
+        <is>
+          <t>Tanner Creek original (Schulz)</t>
+        </is>
+      </c>
+      <c r="C73" s="77" t="n">
+        <v>272</v>
+      </c>
+      <c r="D73" s="77" t="n"/>
+      <c r="E73" s="37" t="inlineStr">
+        <is>
+          <t>DENIED 2018</t>
+        </is>
+      </c>
+      <c r="F73" s="37" t="n"/>
+      <c r="G73" s="37" t="inlineStr">
+        <is>
           <t>Waltman Ln; corridor later approved as phased Tanner Creek (280 apts, CBH) — on watch list.</t>
         </is>
       </c>
-      <c r="H72" s="37" t="inlineStr">
+      <c r="H73" s="37" t="inlineStr">
         <is>
           <t>Meridian records</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="B73" t="inlineStr">
+    <row r="74">
+      <c r="B74" t="inlineStr">
         <is>
           <t>(pattern read)</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
+      <c r="G74" t="inlineStr">
         <is>
           <t>Council kills big MF at retail/employment nodes (protective for subject); denial is often round one — Rolling Hill/Centrepoint/Union 93/Tanner Creek all returned in new form; Magic View enclave killed senior/MF 3x; ~2,100 units died in-ring 2024-2025. Dormant-but-entitled deals (Records #38, Victory Flats #41, Ascent #46, 12548 #45, OZ #47) remain in the chart, NOT here. Syringa #40 is contested-live.</t>
         </is>
       </c>
     </row>
-    <row r="74"/>
-    <row r="75">
-      <c r="B75" s="86" t="inlineStr">
+    <row r="75"/>
+    <row r="76">
+      <c r="B76" s="86" t="inlineStr">
         <is>
           <t>SHADOW WATCH — ADDED AUG 14 2026 (agent sweep)</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="B76" s="37" t="inlineStr">
-        <is>
-          <t>Apex Zenith (Brighton) — Lake Hazel &amp; Meridian Rd</t>
-        </is>
-      </c>
-      <c r="C76" s="77" t="n"/>
-      <c r="D76" s="77" t="n"/>
-      <c r="E76" s="37" t="n"/>
-      <c r="F76" s="37" t="n"/>
-      <c r="G76" s="37" t="inlineStr">
-        <is>
-          <t>AUG 2026 SWEEP: Annexation/rezone/DA approved 4-1 Jan 2025; application references MF units; Costco portion under construction (Aug 2026 opening target). Southern ring edge (~4 mi); MF phases undated.</t>
-        </is>
-      </c>
-      <c r="H76" s="37" t="inlineStr">
-        <is>
-          <t>BoiseDev / Meridian records</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="37" t="inlineStr">
         <is>
-          <t>Victory &amp; Ten Mile mixed-use pre-app (~142 ac)</t>
+          <t>Apex Zenith (Brighton) — Lake Hazel &amp; Meridian Rd</t>
         </is>
       </c>
       <c r="C77" s="77" t="n"/>
@@ -9687,10 +9706,31 @@
       <c r="F77" s="37" t="n"/>
       <c r="G77" s="37" t="inlineStr">
         <is>
+          <t>AUG 2026 SWEEP: Annexation/rezone/DA approved 4-1 Jan 2025; application references MF units; Costco portion under construction (Aug 2026 opening target). Southern ring edge (~4 mi); MF phases undated.</t>
+        </is>
+      </c>
+      <c r="H77" s="37" t="inlineStr">
+        <is>
+          <t>BoiseDev / Meridian records</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="37" t="inlineStr">
+        <is>
+          <t>Victory &amp; Ten Mile mixed-use pre-app (~142 ac)</t>
+        </is>
+      </c>
+      <c r="C78" s="77" t="n"/>
+      <c r="D78" s="77" t="n"/>
+      <c r="E78" s="37" t="n"/>
+      <c r="F78" s="37" t="n"/>
+      <c r="G78" s="37" t="inlineStr">
+        <is>
           <t>AUG 2026 SWEEP: Oct 2025 pre-application concept (Mark Bottles RE / West Ada SD land) with a second housing product plausibly attached/MF; no formal file yet (~2.9 mi).</t>
         </is>
       </c>
-      <c r="H77" s="37" t="inlineStr">
+      <c r="H78" s="37" t="inlineStr">
         <is>
           <t>Oct 2025 reporting</t>
         </is>

</xml_diff>

<commit_message>
Vanguard Village moved UC→Proposed (#33); map gains per-bucket toggle layers
- Chart: UC now 4 properties/661u, Proposed 16/4,494u; renumbered #28-47;
  S&A UC block rewritten to 4 slots, Vanguard added to pipeline block
  (Bear+Base); static UC-vs-CoStar note updated
- Map: pins grouped into toggleable Leaflet overlay layers (checkbox panel);
  renumbered to match

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CQcHG3mGNNEuNdk4jQMCJB
</commit_message>
<xml_diff>
--- a/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
+++ b/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
@@ -893,7 +893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:M61"/>
+  <dimension ref="A2:M61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="79" min="1" max="1"/>
@@ -2198,7 +2198,7 @@
       <c r="B36" s="16" t="n"/>
       <c r="C36" s="81" t="inlineStr">
         <is>
-          <t>UNDER CONSTRUCTION (5 properties, 1,213 units)</t>
+          <t>UNDER CONSTRUCTION (4 properties, 661 units)</t>
         </is>
       </c>
     </row>
@@ -2334,11 +2334,11 @@
       </c>
       <c r="C40" s="18" t="inlineStr">
         <is>
-          <t>Vanguard Village</t>
+          <t>Centrepoint</t>
         </is>
       </c>
       <c r="D40" s="19" t="n">
-        <v>552</v>
+        <v>213</v>
       </c>
       <c r="E40" s="17" t="inlineStr">
         <is>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="H40" s="18" t="inlineStr">
         <is>
-          <t>Endurance Holdings / Challenger Development (CBH)</t>
+          <t>Privately Owned</t>
         </is>
       </c>
       <c r="I40" s="22" t="n">
-        <v>4.3</v>
+        <v>2.9</v>
       </c>
       <c r="J40" s="17" t="inlineStr">
         <is>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="K40" s="18" t="inlineStr">
         <is>
-          <t>Developer: Endurance Holdings LLC + Challenger Development Inc (Corey Barton/CBH org). Evolved from 2022 "Vanguard Commons" 432u filing. UC per CoStar (=its entire 5-mi UC series, 552u) but NO C-MULTI permit found in Meridian public reports 2025-26 — VERIFY construction status before relying on Q1 2028 delivery.</t>
+          <t>RealPage pipeline (not yet in CoStar); Diligence: under construction - revived; permits issuing 2026</t>
         </is>
       </c>
       <c r="M40">
@@ -2374,59 +2374,59 @@
         <v/>
       </c>
     </row>
-    <row r="41">
-      <c r="B41" s="17" t="n">
+    <row r="41"/>
+    <row r="42">
+      <c r="B42" s="23" t="n"/>
+      <c r="C42" s="83" t="inlineStr">
+        <is>
+          <t>PROPOSED (16 properties, 4,494 units)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="24" t="n">
         <v>32</v>
       </c>
-      <c r="C41" s="18" t="inlineStr">
-        <is>
-          <t>Centrepoint</t>
-        </is>
-      </c>
-      <c r="D41" s="19" t="n">
-        <v>213</v>
-      </c>
-      <c r="E41" s="17" t="inlineStr">
-        <is>
-          <t>Q1 2028</t>
-        </is>
-      </c>
-      <c r="F41" s="20" t="n"/>
-      <c r="G41" s="21" t="inlineStr">
+      <c r="C43" s="25" t="inlineStr">
+        <is>
+          <t>Outer Banks Apartments</t>
+        </is>
+      </c>
+      <c r="D43" s="26" t="n">
+        <v>516</v>
+      </c>
+      <c r="E43" s="24" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="n"/>
+      <c r="G43" s="28" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H41" s="18" t="inlineStr">
-        <is>
-          <t>Privately Owned</t>
-        </is>
-      </c>
-      <c r="I41" s="22" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="J41" s="17" t="inlineStr">
-        <is>
-          <t>Mid-Rise</t>
-        </is>
-      </c>
-      <c r="K41" s="18" t="inlineStr">
-        <is>
-          <t>RealPage pipeline (not yet in CoStar); Diligence: under construction - revived; permits issuing 2026</t>
-        </is>
-      </c>
-      <c r="M41">
-        <f>IFERROR(VALUE(RIGHT(E41,4))*4+MATCH(LEFT(E41,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42"/>
-    <row r="43">
-      <c r="B43" s="23" t="n"/>
-      <c r="C43" s="83" t="inlineStr">
-        <is>
-          <t>PROPOSED (15 properties, 3,942 units)</t>
-        </is>
+      <c r="H43" s="25" t="inlineStr">
+        <is>
+          <t>Elk Ventures</t>
+        </is>
+      </c>
+      <c r="I43" s="29" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="J43" s="24" t="inlineStr">
+        <is>
+          <t>Garden</t>
+        </is>
+      </c>
+      <c r="K43" s="25" t="inlineStr">
+        <is>
+          <t>Audit find Aug 2026: 2024 CUP (364 apts/126 flats/26 TH, 19.34 ac R-40/C-C, SW Franklin &amp; Ten Mile); groundbreaking expected 2026, first units summer 2027 (Statesman); Diligence: proposed - near-UC</t>
+        </is>
+      </c>
+      <c r="M43">
+        <f>IFERROR(VALUE(RIGHT(E43,4))*4+MATCH(LEFT(E43,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -2435,15 +2435,15 @@
       </c>
       <c r="C44" s="25" t="inlineStr">
         <is>
-          <t>Outer Banks Apartments</t>
+          <t>Vanguard Village</t>
         </is>
       </c>
       <c r="D44" s="26" t="n">
-        <v>516</v>
+        <v>552</v>
       </c>
       <c r="E44" s="24" t="inlineStr">
         <is>
-          <t>Q4 2027</t>
+          <t>Q1 2028</t>
         </is>
       </c>
       <c r="F44" s="27" t="n"/>
@@ -2454,20 +2454,20 @@
       </c>
       <c r="H44" s="25" t="inlineStr">
         <is>
-          <t>Elk Ventures</t>
+          <t>Endurance Holdings / Challenger Development (CBH)</t>
         </is>
       </c>
       <c r="I44" s="29" t="n">
-        <v>3.3</v>
+        <v>4.3</v>
       </c>
       <c r="J44" s="24" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K44" s="25" t="inlineStr">
         <is>
-          <t>Audit find Aug 2026: 2024 CUP (364 apts/126 flats/26 TH, 19.34 ac R-40/C-C, SW Franklin &amp; Ten Mile); groundbreaking expected 2026, first units summer 2027 (Statesman); Diligence: proposed - near-UC</t>
+          <t>Moved from UC to PROPOSED (analyst call Aug 2026): CoStar carries it UC (Q1 2028) but no C-MULTI permit found in Meridian public reports and no groundbreaking press. Developer: Endurance Holdings/Challenger Development (CBH org); ex-"Vanguard Commons" 432u (2022).</t>
         </is>
       </c>
       <c r="M44">
@@ -3104,6 +3104,7 @@
       </c>
     </row>
     <row r="59"/>
+    <row r="60"/>
     <row r="61">
       <c r="B61" s="84" t="inlineStr">
         <is>
@@ -3131,7 +3132,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:Z75"/>
+  <dimension ref="A1:Z75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="1"/>
   <cols>
     <col width="2.44140625" customWidth="1" style="79" min="1" max="1"/>
@@ -3253,15 +3254,15 @@
         <v>0.95</v>
       </c>
       <c r="R6" s="37">
-        <f>'Competitive Analysis'!C41</f>
+        <f>'Competitive Analysis'!C37</f>
         <v/>
       </c>
       <c r="S6" s="38">
-        <f>'Competitive Analysis'!D41</f>
+        <f>'Competitive Analysis'!D37</f>
         <v/>
       </c>
       <c r="T6" s="39">
-        <f>'Competitive Analysis'!E41</f>
+        <f>'Competitive Analysis'!E37</f>
         <v/>
       </c>
       <c r="V6">
@@ -3315,15 +3316,15 @@
         <v>425</v>
       </c>
       <c r="R8" s="37">
-        <f>'Competitive Analysis'!C37</f>
+        <f>'Competitive Analysis'!C39</f>
         <v/>
       </c>
       <c r="S8" s="38">
-        <f>'Competitive Analysis'!D37</f>
+        <f>'Competitive Analysis'!D39</f>
         <v/>
       </c>
       <c r="T8" s="39">
-        <f>'Competitive Analysis'!E37</f>
+        <f>'Competitive Analysis'!E39</f>
         <v/>
       </c>
       <c r="V8">
@@ -3344,26 +3345,11 @@
       <c r="C9" s="41" t="n">
         <v>850</v>
       </c>
-      <c r="R9" s="37">
-        <f>'Competitive Analysis'!C39</f>
-        <v/>
-      </c>
-      <c r="S9" s="38">
-        <f>'Competitive Analysis'!D39</f>
-        <v/>
-      </c>
-      <c r="T9" s="39">
-        <f>'Competitive Analysis'!E39</f>
-        <v/>
-      </c>
-      <c r="V9">
-        <f>IFERROR(VALUE(RIGHT(T9,4))*4+MATCH(LEFT(T9,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
-        <v/>
-      </c>
-      <c r="W9">
-        <f>IF(V9="","",IF(V9&lt;=$Z$1,0,MAX(1,INT((V9-$Z$2)/4)+1)))</f>
-        <v/>
-      </c>
+      <c r="R9" s="37" t="inlineStr"/>
+      <c r="S9" s="38" t="inlineStr"/>
+      <c r="T9" s="39" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
     </row>
     <row r="10" ht="14.4" customHeight="1" s="79">
       <c r="B10" s="32" t="inlineStr">
@@ -3744,27 +3730,27 @@
         <v/>
       </c>
       <c r="J19" s="47">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,1)+SUMIFS($S$13:$S$27,$W$13:$W$27,1,$X$13:$X$27,1)</f>
+        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,1)+SUMIFS($S$13:$S$28,$W$13:$W$28,1,$X$13:$X$28,1)</f>
         <v/>
       </c>
       <c r="K19" s="47">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,2)+SUMIFS($S$13:$S$27,$W$13:$W$27,2,$X$13:$X$27,1)</f>
+        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,2)+SUMIFS($S$13:$S$28,$W$13:$W$28,2,$X$13:$X$28,1)</f>
         <v/>
       </c>
       <c r="L19" s="47">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,3)+SUMIFS($S$13:$S$27,$W$13:$W$27,3,$X$13:$X$27,1)</f>
+        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,3)+SUMIFS($S$13:$S$28,$W$13:$W$28,3,$X$13:$X$28,1)</f>
         <v/>
       </c>
       <c r="M19" s="47">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,4)+SUMIFS($S$13:$S$27,$W$13:$W$27,4,$X$13:$X$27,1)</f>
+        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,4)+SUMIFS($S$13:$S$28,$W$13:$W$28,4,$X$13:$X$28,1)</f>
         <v/>
       </c>
       <c r="N19" s="47">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,5)+SUMIFS($S$13:$S$27,$W$13:$W$27,5,$X$13:$X$27,1)</f>
+        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,5)+SUMIFS($S$13:$S$28,$W$13:$W$28,5,$X$13:$X$28,1)</f>
         <v/>
       </c>
       <c r="O19" s="47">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,6)+SUMIFS($S$13:$S$27,$W$13:$W$27,6,$X$13:$X$27,1)</f>
+        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,6)+SUMIFS($S$13:$S$28,$W$13:$W$28,6,$X$13:$X$28,1)</f>
         <v/>
       </c>
       <c r="R19" s="37" t="inlineStr">
@@ -4435,6 +4421,36 @@
       </c>
       <c r="O28" s="56">
         <f>IFERROR((O23-O25)/O23,"")</f>
+        <v/>
+      </c>
+      <c r="R28" s="37" t="inlineStr">
+        <is>
+          <t>Vanguard Village</t>
+        </is>
+      </c>
+      <c r="S28" s="38" t="n">
+        <v>552</v>
+      </c>
+      <c r="T28" s="43" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="U28" s="43" t="inlineStr">
+        <is>
+          <t>Bear+Base</t>
+        </is>
+      </c>
+      <c r="V28">
+        <f>IFERROR(VALUE(RIGHT(T28,4))*4+MATCH(LEFT(T28,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
+      </c>
+      <c r="W28">
+        <f>IF(V28="","",IF(V28&lt;=$Z$1,0,MAX(1,INT((V28-$Z$2)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X28">
+        <f>IF(U28="All",1,IF(U28="Bear+Base",IF($Z$3&gt;=2,1,0),IF(U28="Bear only",IF($Z$3&gt;=3,1,0),0)))</f>
         <v/>
       </c>
     </row>
@@ -5380,7 +5396,7 @@
       </c>
       <c r="E68" s="73" t="inlineStr">
         <is>
-          <t>1,213 / 552</t>
+          <t>661 / 552 (Vanguard 552u moved to Proposed pending permit verification)</t>
         </is>
       </c>
     </row>
@@ -7051,7 +7067,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>UNDER CONSTRUCTION</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="H29" s="75" t="n"/>
@@ -7072,7 +7088,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Aug 2026: developer = Endurance Holdings/Challenger (CBH); ex-Vanguard Commons 432u (2022); CoStar UC flag unconfirmed by city permit record — verify</t>
+          <t>Aug 2026: developer = Endurance Holdings/Challenger (CBH); ex-Vanguard Commons 432u (2022); CoStar UC flag unconfirmed by city permit record — verify | Moved UC→PROPOSED Aug 2026 (permit unverified)</t>
         </is>
       </c>
     </row>
@@ -7842,7 +7858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="B1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="2.44140625" customWidth="1" style="79" min="1" max="1"/>
@@ -8787,7 +8803,7 @@
       </c>
       <c r="E35" s="37" t="inlineStr">
         <is>
-          <t>under construction per CoStar - VERIFY (no city permit found)</t>
+          <t>proposed - moved from UC (analyst call): CoStar UC flag unconfirmed by permits</t>
         </is>
       </c>
       <c r="F35" s="37" t="n"/>

</xml_diff>

<commit_message>
IC-ready cleanup: owners on every pipeline row, conclusion-only notes, detail moved to Diligence
- Owner/developer added for all 16 pipeline deals + the 4 other UC rows (Elk Ventures,
  Endurance/Challenger, Hawkins x2, Pacific+Ahlquist, Kal Pacific, Assemble, Brighton,
  GFI Meridian, Welltower, DRB, Quarterra/Baron, Hook Family Trust, MVRK, J. Fisher,
  Shannon Robnett; 12565 W Fairview sponsor is genuinely unverified)
- Notes column rewritten to the IC conclusion only (1-2 lines); full evidence, timelines,
  file numbers, corrections and sources pushed to the Diligence tab
- Restored Outer Banks units (516 = 364 apts + 126 flats + 26 TH) lost in the row move
- Footnote now explains the notes/diligence split and the probability basis
- Fixed a stale merged range left by an earlier row insert

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CQcHG3mGNNEuNdk4jQMCJB
</commit_message>
<xml_diff>
--- a/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
+++ b/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
@@ -288,7 +288,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -507,6 +507,21 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -909,10 +924,10 @@
     <col width="11.44140625" customWidth="1" style="79" min="5" max="5"/>
     <col width="10" customWidth="1" style="79" min="6" max="6"/>
     <col width="13" customWidth="1" style="79" min="7" max="7"/>
-    <col width="22" customWidth="1" style="79" min="8" max="8"/>
+    <col width="30" customWidth="1" style="79" min="8" max="8"/>
     <col width="11" customWidth="1" style="79" min="9" max="9"/>
     <col width="14" customWidth="1" style="79" min="10" max="10"/>
-    <col width="30" customWidth="1" style="79" min="11" max="11"/>
+    <col width="62" customWidth="1" style="79" min="11" max="11"/>
     <col hidden="1" width="13" customWidth="1" style="79" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -1963,6 +1978,7 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="B29" s="9" t="n"/>
       <c r="C29" s="85" t="inlineStr">
@@ -2205,6 +2221,7 @@
         <v/>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="B36" s="16" t="n"/>
       <c r="C36" s="81" t="inlineStr">
@@ -2236,7 +2253,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H37" s="18" t="inlineStr">
+      <c r="H37" s="91" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2249,7 +2266,11 @@
           <t>Garden</t>
         </is>
       </c>
-      <c r="K37" s="18" t="n"/>
+      <c r="K37" s="91" t="inlineStr">
+        <is>
+          <t>Phase II of the delivered South Ridge I (476u, 2022) at the same Grand Fork Way site.</t>
+        </is>
+      </c>
       <c r="M37">
         <f>IFERROR(VALUE(RIGHT(E37,4))*4+MATCH(LEFT(E37,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
@@ -2278,18 +2299,18 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H38" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H38" s="91" t="inlineStr">
+        <is>
+          <t>J. Fisher Companies</t>
         </is>
       </c>
       <c r="I38" s="22" t="n">
         <v>4.9</v>
       </c>
       <c r="J38" s="17" t="n"/>
-      <c r="K38" s="18" t="inlineStr">
-        <is>
-          <t>Analyst-sourced deal (not in CoStar/RealPage); Diligence: under construction</t>
+      <c r="K38" s="91" t="inlineStr">
+        <is>
+          <t>Broke ground Oct 2025. 100% income-restricted (50-80% AMI, incl. 21 Our Path Home units), $70M — limited overlap with the subject at $1,796.</t>
         </is>
       </c>
       <c r="M38">
@@ -2320,18 +2341,18 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H39" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H39" s="91" t="inlineStr">
+        <is>
+          <t>Shannon Robnett Industries</t>
         </is>
       </c>
       <c r="I39" s="22" t="n">
         <v>3.5</v>
       </c>
       <c r="J39" s="17" t="n"/>
-      <c r="K39" s="18" t="inlineStr">
-        <is>
-          <t>Analyst-sourced deal (not in CoStar/RealPage); Diligence: under construction</t>
+      <c r="K39" s="91" t="inlineStr">
+        <is>
+          <t>Phased garden/rowhouse community at Ustick &amp; Venable; early buildings leasing, three new 24-plex permits issued June 2025.</t>
         </is>
       </c>
       <c r="M39">
@@ -2362,9 +2383,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H40" s="18" t="inlineStr">
-        <is>
-          <t>Privately Owned</t>
+      <c r="H40" s="91" t="inlineStr">
+        <is>
+          <t>Studio PBA (market-rate replacement)</t>
         </is>
       </c>
       <c r="I40" s="22" t="n">
@@ -2375,9 +2396,9 @@
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K40" s="18" t="inlineStr">
-        <is>
-          <t>RealPage pipeline (not yet in CoStar); Diligence: under construction - revived; permits issuing 2026</t>
+      <c r="K40" s="91" t="inlineStr">
+        <is>
+          <t>213u market-rate approved Dec 2025 REPLACING DevCo's 239u affordable plan, which died in 2025 when its LIHTC financing collapsed. Permits issuing 2026.</t>
         </is>
       </c>
       <c r="M40">
@@ -2394,7 +2415,9 @@
           <t>Outer Banks Apartments</t>
         </is>
       </c>
-      <c r="D41" s="19" t="n"/>
+      <c r="D41" s="19" t="n">
+        <v>516</v>
+      </c>
       <c r="E41" s="17" t="inlineStr">
         <is>
           <t>Q1 2028</t>
@@ -2402,12 +2425,22 @@
       </c>
       <c r="F41" s="20" t="n"/>
       <c r="G41" s="21" t="n"/>
-      <c r="H41" s="18" t="n"/>
-      <c r="I41" s="22" t="n"/>
-      <c r="J41" s="17" t="n"/>
-      <c r="K41" s="18" t="inlineStr">
-        <is>
-          <t>PERMITTED: C-MULTI-2025-0023/-0024 + a third issued 6/17/2026 (Bldgs A/B/C, S Tallac Ln); GC Perryman Construction Mgmt; owner 10 Mile Franklin LLC. Current entitlement is H-2024-0026 (2021 CUP lapsed ~Dec 2023). ONLY permitted deal in the ring.</t>
+      <c r="H41" s="91" t="inlineStr">
+        <is>
+          <t>Elk Ventures (10 Mile Franklin LLC)</t>
+        </is>
+      </c>
+      <c r="I41" s="22" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="J41" s="17" t="inlineStr">
+        <is>
+          <t>Garden</t>
+        </is>
+      </c>
+      <c r="K41" s="91" t="inlineStr">
+        <is>
+          <t>BUILDING NOW — the only permitted deal in the ring. 3 of ~50 bldgs permitted 6/17/26; first units Q4 27-Q2 28, full 516u into 2029-30.</t>
         </is>
       </c>
       <c r="L41" s="90" t="n">
@@ -2418,6 +2451,7 @@
         <v/>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="B43" s="23" t="n"/>
       <c r="C43" s="83" t="inlineStr">
@@ -2449,9 +2483,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H44" s="25" t="inlineStr">
-        <is>
-          <t>Endurance Holdings / Challenger Development (CBH)</t>
+      <c r="H44" s="92" t="inlineStr">
+        <is>
+          <t>Endurance Holdings / Challenger Dev (CBH)</t>
         </is>
       </c>
       <c r="I44" s="29" t="n">
@@ -2462,9 +2496,9 @@
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K44" s="25" t="inlineStr">
-        <is>
-          <t>CORRECTION: CoStar UC flag is bleed-over from the $50.7M Life Time club (C-NEW-2026-0003) on a commercial lot in the same plat. R-15 parcel raw, unplatted, ZERO permits across 5 weekly + Jan-2026 monthly reports. CUP likely lapsed ~Jul 2024; DA absorbed into the commercial-first District at Ten Mile agreement.</t>
+      <c r="K44" s="92" t="inlineStr">
+        <is>
+          <t>NOT under construction — CoStar flag is wrong. Raw land, zero permits, CUP likely lapsed ~Jul 2024. Treat as dormant paper.</t>
         </is>
       </c>
       <c r="L44" s="90" t="n">
@@ -2498,18 +2532,18 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H45" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H45" s="92" t="inlineStr">
+        <is>
+          <t>Hawkins Companies</t>
         </is>
       </c>
       <c r="I45" s="29" t="n">
         <v>3.4</v>
       </c>
       <c r="J45" s="24" t="n"/>
-      <c r="K45" s="25" t="inlineStr">
-        <is>
-          <t>174u approved by Boise Council 9/10/2024; 162 per DRH24-00090 redesign. ~4.2 of 6.1 ac cleared/graded. CUP commencement appears to expire ~9/10/2026, no extension found; approved 3-2 over a P&amp;Z denial rec.</t>
+      <c r="K45" s="92" t="inlineStr">
+        <is>
+          <t>Real dirt moved (~4.2 of 6.1 ac graded) but the CUP clock appears to expire ~9/10/26 with no extension found. Watch for a lapse or extension filing.</t>
         </is>
       </c>
       <c r="L45" s="90" t="n">
@@ -2543,18 +2577,18 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H46" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H46" s="92" t="inlineStr">
+        <is>
+          <t>Pacific Companies + Ahlquist (Gray Owl)</t>
         </is>
       </c>
       <c r="I46" s="29" t="n">
         <v>1.9</v>
       </c>
       <c r="J46" s="24" t="n"/>
-      <c r="K46" s="25" t="inlineStr">
-        <is>
-          <t>UNENTITLED: the Mar-2020 CUP covered a different program (385u, no office/hotel). Current ~250u + 120k sf office + 32k sf retail has NO filed application as of Aug 2026 ("very nascent design"). Sponsors Ahlquist + Pacific Cos; $6.77M foreclosure basis.</t>
+      <c r="K46" s="92" t="inlineStr">
+        <is>
+          <t>Strong sponsors and a cheap basis ($6.77M at foreclosure) — but NO application filed as of Aug 2026 and the program is unentitled. 2030 at best.</t>
         </is>
       </c>
       <c r="L46" s="90" t="n">
@@ -2588,9 +2622,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H47" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H47" s="92" t="inlineStr">
+        <is>
+          <t>Kal Pacific (Don Veasy)</t>
         </is>
       </c>
       <c r="I47" s="29" t="n">
@@ -2601,9 +2635,9 @@
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K47" s="25" t="inlineStr">
-        <is>
-          <t>224u version has NO CUP, no DA, no design-review approval, no confirmed hearing. Only approval this site ever had is the 2021 DA for 136u, never permitted, which must be terminated by Council. File no. PLN26-00493 unverified.</t>
+      <c r="K47" s="92" t="inlineStr">
+        <is>
+          <t>No entitlement for the 224u program — the only approval this site ever had was a 2021 DA for 136u that was never permitted. Post-2031.</t>
         </is>
       </c>
       <c r="L47" s="90" t="n">
@@ -2637,18 +2671,18 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H48" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H48" s="92" t="inlineStr">
+        <is>
+          <t>Assemble Management</t>
         </is>
       </c>
       <c r="I48" s="29" t="n">
         <v>1</v>
       </c>
       <c r="J48" s="24" t="n"/>
-      <c r="K48" s="25" t="inlineStr">
-        <is>
-          <t>200u/~19,517 sf confirmed at the 5/19/2026 council hearing. Cleanest entitlement in the ring, no lapse risk until ~2028. RISK: land was LOI-stage not closed at approval; View Circle collector unfunded (staff: "may never be constructed"); single unsignaled RI/RO access for 200u.</t>
+      <c r="K48" s="92" t="inlineStr">
+        <is>
+          <t>Freshest entitlement in the ring (approved 5-1 on 5/19/26, no lapse risk to ~2028) — but land was LOI-stage, not closed, and the access road is unfunded.</t>
         </is>
       </c>
       <c r="L48" s="90" t="n">
@@ -2682,9 +2716,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H49" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H49" s="92" t="inlineStr">
+        <is>
+          <t>Brighton Development</t>
         </is>
       </c>
       <c r="I49" s="29" t="n">
@@ -2695,9 +2729,9 @@
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K49" s="25" t="inlineStr">
-        <is>
-          <t>ENTITLEMENT LIKELY LAPSED: CUP H-2022-0008 base clock expired ~Apr/May 2024; outside limit even with max Director TEC was ~Apr/May 2026 — passed. No TECC in any 2022-2026 council agenda. Parcel S1104347006 still PROPCODE F, TOTALVALUE $21,000. Re-entitlement required.</t>
+      <c r="K49" s="92" t="inlineStr">
+        <is>
+          <t>ENTITLEMENT LAPSED. Base clock ran out ~Apr/May 2024 and even a maximum extension expired ~Apr/May 2026. Requires full re-entitlement.</t>
         </is>
       </c>
       <c r="L49" s="90" t="n">
@@ -2731,9 +2765,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H50" s="25" t="inlineStr">
-        <is>
-          <t>TGI Corp</t>
+      <c r="H50" s="92" t="inlineStr">
+        <is>
+          <t>GFI Meridian Investments (Trevor Gasser)</t>
         </is>
       </c>
       <c r="I50" s="29" t="n">
@@ -2744,9 +2778,9 @@
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K50" s="25" t="inlineStr">
-        <is>
-          <t>Applicant is GFI Meridian Investments LLC (NOT TGI Corp); engineer KM Engineering. Approved unanimously 11/19/2024. Developer on record: commercial first, residential 5-7 yrs out; commercial still at pad-leasing stage. CUP commencement lapses ~11/19/2026, no TEC found. Ten Mile at LOS F.</t>
+      <c r="K50" s="92" t="inlineStr">
+        <is>
+          <t>Developer says residential is 5-7 years out; commercial builds first and is only at pad-leasing stage. CUP lapses ~11/19/26.</t>
         </is>
       </c>
       <c r="L50" s="90" t="n">
@@ -2780,9 +2814,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H51" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H51" s="92" t="inlineStr">
+        <is>
+          <t>Hawkins Companies</t>
         </is>
       </c>
       <c r="I51" s="29" t="n">
@@ -2793,9 +2827,9 @@
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K51" s="25" t="inlineStr">
-        <is>
-          <t>NOT ENTITLED: unanimous P&amp;Z denial rec 4/2/2026, council remand 6/16/2026, 8+ months and 6+ hearings. Staff objection (south parcel 68% residential vs 50% cap) only partly cured. 8/6/2026 re-hearing outcome unpublished. 302u is Phase 1 only; combined plan ~400-423 homes.</t>
+      <c r="K51" s="92" t="inlineStr">
+        <is>
+          <t>NOT entitled. Unanimous P&amp;Z denial rec 4/2/26, council remand 6/16/26, re-heard 8/6/26 with the outcome still unpublished. 302u is Phase 1 only.</t>
         </is>
       </c>
       <c r="L51" s="90" t="n">
@@ -2829,9 +2863,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H52" s="25" t="inlineStr">
-        <is>
-          <t>Welltower Inc.</t>
+      <c r="H52" s="92" t="inlineStr">
+        <is>
+          <t>Welltower Inc (Layton Construction)</t>
         </is>
       </c>
       <c r="I52" s="29" t="n">
@@ -2842,9 +2876,9 @@
           <t>Townhome</t>
         </is>
       </c>
-      <c r="K52" s="25" t="inlineStr">
-        <is>
-          <t>WORSE THAN RECORDED: the Jan-2024 two-year extension ALSO lapsed; a SECOND extension request (PUD21-00062) hit the Boise P&amp;Z docket 5/4/2026, outcome unknown. Land owned outright ($12M 2021, assessed $9.1M). Sponsor is a healthcare REIT — MF is non-core.</t>
+      <c r="K52" s="92" t="inlineStr">
+        <is>
+          <t>Extension-as-life-support: the Jan-2024 extension ALSO lapsed and a SECOND request was docketed 5/4/26. Healthcare REIT owner; MF is non-core.</t>
         </is>
       </c>
       <c r="L52" s="90" t="n">
@@ -2878,9 +2912,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H53" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H53" s="92" t="inlineStr">
+        <is>
+          <t>UNVERIFIED — not publicly disclosed</t>
         </is>
       </c>
       <c r="I53" s="29" t="n">
@@ -2891,9 +2925,9 @@
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K53" s="25" t="inlineStr">
-        <is>
-          <t>Shows "Entitled" on Boise's live tracker; second design review DRH26-00124. BUT developer/owner identity unknown, no permit 16 months post concept review, and 4-5 story structured-parking product needs rents far above the garden hurdle. Prior AutoNation entitlement here also lapsed.</t>
+      <c r="K53" s="92" t="inlineStr">
+        <is>
+          <t>Shows "Entitled" on Boise's tracker but the developer is unknown and there is no permit 16 months post concept review. Structured-parking product needs rents well above the garden hurdle.</t>
         </is>
       </c>
       <c r="L53" s="90" t="n">
@@ -2927,18 +2961,18 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H54" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H54" s="92" t="inlineStr">
+        <is>
+          <t>DRB Investments (Matt Baker)</t>
         </is>
       </c>
       <c r="I54" s="29" t="n">
         <v>1.4</v>
       </c>
       <c r="J54" s="24" t="n"/>
-      <c r="K54" s="25" t="inlineStr">
-        <is>
-          <t>CUP current to ~10/21/2027. Developer guidance: groundbreaking "2027 or later," TOWNHOMES FIRST not the 270u. Podium/underground parking basis well above the garden benchmark. Same MDA carries up to ~848-900 apts + ~30-35 TH over 10-12 yrs (~$1B) — see shadow row.</t>
+      <c r="K54" s="92" t="inlineStr">
+        <is>
+          <t>CUP current to ~10/21/27 and the sponsor has real credibility (built Dovetail here) — but its own guidance is townhomes FIRST, groundbreaking "2027 or later."</t>
         </is>
       </c>
       <c r="L54" s="90" t="n">
@@ -2972,9 +3006,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H55" s="25" t="inlineStr">
-        <is>
-          <t>Quarterra</t>
+      <c r="H55" s="92" t="inlineStr">
+        <is>
+          <t>Quarterra (TPG-controlled); land: Baron Properties</t>
         </is>
       </c>
       <c r="I55" s="29" t="n">
@@ -2985,9 +3019,9 @@
           <t>Garden</t>
         </is>
       </c>
-      <c r="K55" s="25" t="inlineStr">
-        <is>
-          <t>EARLIEST-STAGE DEAL: no application, no H-file, no hearing. QUARTERRA DOES NOT OWN THE LAND — Baron Properties still marketing it. 18 u/ac needs a discretionary CPAM vs a 15 u/ac cap. 250u (204 apt + 46 TH) is the plan of record; 256 is Quarterra internal. Prior Artisan approval was 138 BTR (not 131).</t>
+      <c r="K55" s="92" t="inlineStr">
+        <is>
+          <t>Earliest-stage deal in the pipeline — no application, no H-file, no hearing, AND Quarterra does not own the land (Baron is still trying to sell it).</t>
         </is>
       </c>
       <c r="L55" s="90" t="n">
@@ -3021,9 +3055,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H56" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H56" s="92" t="inlineStr">
+        <is>
+          <t>Hook Family Trust</t>
         </is>
       </c>
       <c r="I56" s="29" t="n">
@@ -3034,9 +3068,9 @@
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K56" s="25" t="inlineStr">
-        <is>
-          <t>LAPSED: PUD commencement deadline ~3/12/2026 passed, no extension ever filed; zero city case activity since 10/23/2023. Owner is a family trust that listed the entitled land 8 days after approval and never found a buyer. Site still earns income as RV storage.</t>
+      <c r="K56" s="92" t="inlineStr">
+        <is>
+          <t>LAPSED — PUD commencement passed ~3/12/26 with no extension ever filed; zero city activity since 10/23/23. Site earns income as RV storage.</t>
         </is>
       </c>
       <c r="L56" s="90" t="n">
@@ -3070,9 +3104,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H57" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H57" s="92" t="inlineStr">
+        <is>
+          <t>MVRK Development (under contract 8/7/26)</t>
         </is>
       </c>
       <c r="I57" s="29" t="n">
@@ -3083,9 +3117,9 @@
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K57" s="25" t="inlineStr">
-        <is>
-          <t>STATUS CHANGE: UNDER CONTRACT ~8/7/2026 after 469 days on market (Crexi/BHHS). Buyer, price, intended use all unknown. The "$5.0M CBRE asking price" we carried could NOT be verified — the live listing is unpriced. Original developer chose to sell rather than build.</t>
+      <c r="K57" s="92" t="inlineStr">
+        <is>
+          <t>UNDER CONTRACT 8/7/26 after 469 days on market — the developer chose to sell rather than build. Buyer and intent unknown.</t>
         </is>
       </c>
       <c r="L57" s="90" t="n">
@@ -3119,9 +3153,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H58" s="25" t="inlineStr">
-        <is>
-          <t>Peak Capital Investments Llc</t>
+      <c r="H58" s="92" t="inlineStr">
+        <is>
+          <t>SOLD 8/7/26 — buyer unknown (was Realm Venture)</t>
         </is>
       </c>
       <c r="I58" s="29" t="n">
@@ -3132,9 +3166,9 @@
           <t>Garden</t>
         </is>
       </c>
-      <c r="K58" s="25" t="inlineStr">
-        <is>
-          <t>STATUS CHANGE: SOLD 8/7/2026 for $1,700,000 (MLS 98949803, list = close). Buyer unknown. CUP MCU-2024-0002 commencement EXPIRES ~10/17/2026 — no extension found. Survived a 2023 denial, redesigned 60u -&gt; 36u.</t>
+      <c r="K58" s="92" t="inlineStr">
+        <is>
+          <t>SOLD 8/7/26 for $1.7M. CUP expires ~10/17/26 — about 8 weeks out — with no extension filed and no sign the new owner is moving to permit.</t>
         </is>
       </c>
       <c r="L58" s="90" t="n">
@@ -3146,10 +3180,11 @@
       </c>
     </row>
     <row r="59"/>
+    <row r="60"/>
     <row r="61">
-      <c r="B61" s="84" t="inlineStr">
-        <is>
-          <t>* 5-Mile radius. Rent ($) = HelloData mix-weighted asking where covered, else market asking (CoStar). Proximity (mi) = straight-line distance from the subject. Est. Delivery drives the Supply &amp; Absorption tab's per-window supply (edit it there or here — they are linked). See the 'Supply &amp; Absorption' tab for the forward supply / absorption / overall-occupancy forecast.</t>
+      <c r="B61" s="95" t="inlineStr">
+        <is>
+          <t>* 5-Mile radius. Rent ($) = HelloData mix-weighted asking where covered, else CoStar market asking. Proximity (mi) = straight-line from the subject. Est. Delivery drives the Supply &amp; Absorption tab. NOTES = the IC conclusion only; full evidence, timelines, file numbers and sources are on the DILIGENCE tab, source reconciliation on the RECONCILIATION LOG. P(deliver by YE2031) is a reasoned probability from the Aug-2026 46-agent deep dive (research/audit_2026-08/pipeline_likelihood_report.md), weighting permits and financing far above entitlement status: 4,494 proposed units -&gt; 1,221 probability-weighted.</t>
         </is>
       </c>
     </row>
@@ -7896,7 +7931,7 @@
     <col width="12" customWidth="1" style="79" min="4" max="4"/>
     <col width="16" customWidth="1" style="79" min="5" max="5"/>
     <col width="14" customWidth="1" style="79" min="6" max="6"/>
-    <col width="50" customWidth="1" style="79" min="7" max="7"/>
+    <col width="110" customWidth="1" style="79" min="7" max="7"/>
     <col width="36" customWidth="1" style="79" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -7991,9 +8026,9 @@
         </is>
       </c>
       <c r="F5" s="37" t="n"/>
-      <c r="G5" s="37" t="inlineStr">
-        <is>
-          <t>DEEP-DIVE VERIFIED 7/16/2026 (all verdicts survived 3-lens adversarial check). CUP H-2022-0008 heard Apr 7 2022 (staff conditioned approval on cutting to ~40 du/ac ≈ 398u vs 472 proposed); NO CZC, permit, extension, or hearing step since, and Meridian permit reports through Apr 2026 show nothing at Records Way. Under Meridian's 2-yr CUP commencement rule the entitlement has very likely expired — would need re-entitlement. Brighton's page has said 'coming soon' for 4+ years while its news feed promotes everything else. Not verifiably dead (no site sale found) — Bear-only, undated.</t>
+      <c r="G5" s="93" t="inlineStr">
+        <is>
+          <t>Brighton Development Inc (Brighton Corporation). 472u urban product at the NE corner of Fairview &amp; Records Way. CUP H-2022-0008 approved ~spring 2022; base 2-year commencement expired ~Apr/May 2024; the outside limit even with a maximum unposted Director TEC was ~Apr/May 2026 — also passed. No TECC appears in any 2022-2026 council agenda. Parcel S1104347006 remains PROPCODE F with TOTALVALUE $21,000 (still assessed as farmland). Brighton still markets "Records" as coming soon but has been publicly silent 4+ years. Deep-pocketed local sponsor with continued site control and an easy re-entitlement path (already C-G, no annexation, no opposition record) — which is why this is 20% and not lower. 5-story podium is the exact product the LTC compression punishes.</t>
         </is>
       </c>
       <c r="H5" s="37" t="inlineStr">
@@ -8105,9 +8140,9 @@
         </is>
       </c>
       <c r="F9" s="37" t="n"/>
-      <c r="G9" s="37" t="inlineStr">
-        <is>
-          <t>DEEP-DIVE VERIFIED 7/16/2026 (all verdicts survived 3-lens adversarial check). Status unchanged and current: P&amp;Z recommended denial Apr 2 2026; council unanimously REMANDED the revised plan (up to 400 homes, more office/retail, ITD right-in/right-out granted on SH-69) back to P&amp;Z on 6/17/2026; no re-hearing outcome as of 7/16/2026 and staff still say revisions don't cure comp-plan inconsistencies. Hawkins still markets the corners as a 'proposed' shopping center. No annexation, plat, or permits — Bear-case only with elevated kill risk; earliest delivery ~2029 if it survives. Land-use dossier SM-12 covers the adjacent block. | AUG 2026 AUDIT: CUP now 302 units on 15.23 ac R-40 inside ~400-home plan; P&amp;Z rec. denial 4/2/26, council remanded 6/17/26, re-heard 8/6/26.</t>
+      <c r="G9" s="93" t="inlineStr">
+        <is>
+          <t>Hawkins Companies (Boise). 302u MF CUP on 15.23 ac R-40 at Meridian Rd/SH-69 &amp; Amity — Phase 1 only; the combined annexation carries ~400-423 homes including 86-101 R-15 apartments/townhomes on the north parcel (shadow, not counted). Process: unanimous P&amp;Z denial recommendation 4/2/2026; Council REMANDED rather than denied 6/16/2026; P&amp;Z re-heard 8/6/2026 — OUTCOME STILL UNPUBLISHED as of 8/15/2026. 8+ months and 6+ hearings so far. Staff core objection (south parcel 68% residential vs a 50% cap) only partly cured by the revision. ITD granted a right-in/right-out SH-69 access June 2026, a genuine positive.</t>
         </is>
       </c>
       <c r="H9" s="37" t="inlineStr">
@@ -8136,9 +8171,9 @@
         </is>
       </c>
       <c r="F10" s="37" t="n"/>
-      <c r="G10" s="37" t="inlineStr">
-        <is>
-          <t>DEEP-DIVE VERIFIED 7/16/2026 (all verdicts survived 3-lens adversarial check). Stale in BOTH directions: the 136u plan got further than believed — $11.2M foundation/podium permit BLD22-03293 was ISSUED 4/5/2024 — but was never built and EXPIRED 3/31/2026 (parcel S1007325725 still vacant land, $2.78M, on the 2026 roll). Then in May/Jun 2026 a NEW filing appeared on the same 2.13-ac MX-3/DA parcel: PLN26-00493 '580 N COLE RD - DRH', a six-story mixed-use building with 200+ apartments (sponsor almost certainly Kal Pacific), at neighborhood-meeting/design-review stage (tracker 6/15/2026). LoopNet listing off-market. Live early-stage ~200u proposal; delivery 2029+; do NOT promote to UC. City separately buying neighboring 709 N Cole for affordable housing. | AUG 2026 AUDIT: unit count raised to 224 per BoiseDev 7/27/26 (Kal Pacific abandons 2021 DA, uses Boise 2023 code).</t>
+      <c r="G10" s="93" t="inlineStr">
+        <is>
+          <t>Kal Pacific (Garden City ID office; principal Don Veasy, Temecula CA) — a small commercial/shopping-center developer, not an MF specialist; Veasy also controls Urban Capital Partners. 224u is the May/Jul 2026 redesign (up from 136u). ENTITLEMENT: no CUP, no DA, no design-review approval, no confirmed hearing date for the 224u version; the recorded 2021 DA for 136u must be terminated by Council first. The 136u version sat in permit "corrections" 16+ months and died. MX-3 under Boise 2023 code has no density cap = an easier procedural path, but Cole Rd is torn up through 2026. File no. PLN26-00493 could NOT be confirmed in any city document — treat as unverified.</t>
         </is>
       </c>
       <c r="H10" s="37" t="inlineStr">
@@ -8169,9 +8204,9 @@
         </is>
       </c>
       <c r="F11" s="37" t="n"/>
-      <c r="G11" s="37" t="inlineStr">
-        <is>
-          <t>DEEP-DIVE VERIFIED 7/16/2026 (all verdicts survived 3-lens adversarial check). Never verifiably advanced past pre-application/neighborhood-meeting stage (Apr 2025); no application, hearing, approval, or permit since — ~15 months of silence. Mar 2026 city permit report shows nothing at the address; absent from BoiseDev's Feb 2026 zoning-year recap of 2025 approvals. AutoNation still owner, site not re-listed. Bear-only shadow. Sits on land-use developable parcel S1109110516.</t>
+      <c r="G11" s="93" t="inlineStr">
+        <is>
+          <t>Developer/owner UNVERIFIED — not disclosed in any public source located. 275u, 4-5 story with structured parking. Shows as "Entitled" on Boise's live daily-updated development tracker; a second design review (DRH26-00124) shows continued engagement. RISK: no permit 16 months after concept review; the site's prior AutoNation entitlement also lapsed (2023); structured-parking product carries a cost basis materially above the $305-322k/unit garden benchmark, so its required rent sits even further above the $2,224/u/mo hurdle. The unknown sponsor is itself the risk.</t>
         </is>
       </c>
       <c r="H11" s="37" t="inlineStr">
@@ -8202,9 +8237,9 @@
         </is>
       </c>
       <c r="F12" s="37" t="n"/>
-      <c r="G12" s="37" t="inlineStr">
-        <is>
-          <t>DEEP-DIVE VERIFIED 7/16/2026 (all verdicts survived 3-lens adversarial check). Built-to-sell entitlement drifting toward dead: PUD approved 3/12/2024 and the site was listed on LoopNet THE SAME WEEK (3/4/2024); listing since pulled with no evidence of sale (Ada Cty roll still bare 5.4-ac commercial parcel, $2.66M). Boise PUD approvals lapse 24 months absent construction =&gt; likely expired ~Mar 2026; no permit through June 2026. Overland RV Storage still operating with active waiting lists (site live; Yelp updated Jun 2026). Bear-only.</t>
+      <c r="G12" s="93" t="inlineStr">
+        <is>
+          <t>Hook Family Trust (filed under case name "HOOK"; trust established 3/11/2003) — a long-time family landowner, no institutional apartment developer involved. 156u. LAPSED: PUD/CAR/DRH approvals from Oct 2023; commencement deadline ~3/12/2026 passed with no extension ever filed; zero city case activity since 10/23/2023. The owner listed the entitled land 8 days after approval and never found a buyer. The site continues to earn income as RV storage, which removes any carrying-cost pressure to develop.</t>
         </is>
       </c>
       <c r="H12" s="37" t="inlineStr">
@@ -8335,9 +8370,9 @@
         </is>
       </c>
       <c r="F17" s="37" t="n"/>
-      <c r="G17" s="37" t="inlineStr">
-        <is>
-          <t>DEEP-DIVE VERIFIED 7/16/2026 (all verdicts survived 3-lens adversarial check). 60u plan never built; entitlement MODIFIED DOWN to 36 units Oct 2024 (MCU-2024-0002, Pivot North; findings adopted 10/17/2024). Owner then listed the 2.39-ac site at $1.7M as a 'fully entitled' OZ development opportunity (IMLS 98949803); listing went PENDING, now off-market as of 7/16/2026 — sale closed or withdrawn, no new owner/permit surfaced; no building permit in Meridian reports. Sponsor Realm's other Meridian project was denied Nov 2024 (winding down). Bear-only at 36u, undated.</t>
+      <c r="G17" s="93" t="inlineStr">
+        <is>
+          <t>Original developer Realm Venture Group (2022-23); the 2024 modification was filed by Pivot North Design (Danielle Stehman) as agent. SOLD 8/7/2026 for $1,700,000 (MLS 98949803 — list price = close price); buyer unknown. 36u = 18 one-bed + 18 two-bed at 15 du/ac in 3 climate-controlled buildings, DOWN from the originally proposed 60u/25 du/ac/8 garden buildings. Site: 1475 E Franklin Rd (SW corner Franklin &amp; Locust Grove), 2.39 ac, R-40, in an Idaho Opportunity Zone. CUP approved 10/17/2024 but its 2-year commencement expires ~10/17/2026 with no extension evidence — and the site changed hands one week before this analysis. This parcel has now failed three times: a 1999 DA for 90+ apartments lapsed, a 60u plan was denied Mar 2023, and the 36u redesign is about to run out of clock.</t>
         </is>
       </c>
       <c r="H17" s="37" t="inlineStr">
@@ -8393,9 +8428,9 @@
         </is>
       </c>
       <c r="F19" s="37" t="n"/>
-      <c r="G19" s="37" t="inlineStr">
-        <is>
-          <t>DEEP-DIVE VERIFIED 7/16/2026 (all verdicts survived 3-lens adversarial check). Approved Mar 2022; real permitting-stage effort followed (submittals, Idaho Power payments, ACHD/Veolia coordination) but Jan 2024 Welltower took a cost-driven TWO-YEAR extension to start construction — that window has now run out with no permit ever issued at 8373 W Victory Rd (city open-data through June 2026). BoiseDev tracker stale since Feb 2022; Welltower still owns. Bear-only; CoStar's Q3 2028 has no support.</t>
+      <c r="G19" s="93" t="inlineStr">
+        <is>
+          <t>Owner Welltower Inc (NYSE: WELL, Toledo OH); developer/applicant Layton Construction (Alex Drecksel). 301u at 8373 W Victory Rd, Boise. Approved Mar 2022. WORSE THAN OUR PRIOR RECORD: the city granted a two-year extension ~Jan 2024, that extension ALSO lapsed, and a SECOND extension request (PUD21-00062) hit the Boise P&amp;Z docket 5/4/2026 with the outcome unknown. Land owned outright ($12M paid 2021; assessed $9.1M, i.e. carried below cost). Sponsor is a healthcare REIT for whom market-rate MF is non-core; sibling project Vista Point (~800u) also sits unbuilt.</t>
         </is>
       </c>
       <c r="H19" s="37" t="inlineStr">
@@ -8451,9 +8486,9 @@
         </is>
       </c>
       <c r="F21" s="37" t="n"/>
-      <c r="G21" s="37" t="inlineStr">
-        <is>
-          <t>DEEP-DIVE VERIFIED 7/16/2026 (all verdicts survived 3-lens adversarial check). Entitlement live (H-2024-0010, Nov 2024) and the COMMERCIAL phase is being marketed (MJPCRE retail pad ground-lease campaign, Nov 2025) — but developer told council residential is 'at least five to seven years out' (~2030-2032) and no residential permits/plats exist through June 2026. IDENTITY WARNING: the June 2026 C-MULTI-2025-0023/24/25 permits at Franklin &amp; Ten Mile are OUTER BANKS (516u, SW corner) — do NOT attribute to Gateway. Bear-only; discard CoStar's Q4 2028.</t>
+      <c r="G21" s="93" t="inlineStr">
+        <is>
+          <t>GFI Meridian Investments LLC (Trevor Gasser, Bountiful UT); site entity GFI - Meridian Investments II LLC; engineer KM Engineering LLP. CORRECTION: our chart carried "TGI Corp" — no such entity appears in any primary source. 390u = 200 1BR + 174 2BR + 16 3BR in six 4-story interior-corridor buildings + five 3-story townhome-style buildings. Site: NE corner Franklin &amp; Ten Mile, 38.99 ac, C-G + R-40, parcel S1211336065 — a DIFFERENT corner and developer from Outer Banks (no double-count). CUP + preliminary plat approved unanimously 11/19/2024. RISK: commencement lapses ~11/19/2026 (~3 months out) with no TEC found; developer stated on the record that residential is 5-7 years out with commercial first, and the commercial is still only at pad-leasing stage; Ten Mile rated LOS F with no widening programmed; 80+ opposition letters on file.</t>
         </is>
       </c>
       <c r="H21" s="37" t="inlineStr">
@@ -8484,9 +8519,9 @@
         </is>
       </c>
       <c r="F22" s="37" t="n"/>
-      <c r="G22" s="37" t="inlineStr">
-        <is>
-          <t>DEEP-DIVE VERIFIED 7/16/2026 (all verdicts survived 3-lens adversarial check). Approved 5-1 Nov 2023 (11880 W Overland Rd, ~3.5 ac); 2.5+ yrs later no permit, no groundbreaking, and MVRK's own projects page still says 'TBD' (checked 7/16/2026). The site is marketed FOR SALE as a 'fully entitled development opportunity' at $4,999,999 with CBRE (MLS 98945418) — sponsor exiting, not building. Feb 2025 ConstructConnect record still 'Design' stage. Bear-only; delivery depends on a hypothetical buyer.</t>
+      <c r="G22" s="93" t="inlineStr">
+        <is>
+          <t>MVRK Development (Denver-based multifamily/condo developer active in Boise). 138u on ~3.5 ac, approved 5-1 Nov 2023. STATUS CHANGE: went under contract ~8/7/2026 after 469 days on market (Crexi/BHHS). The original developer chose to sell rather than build while executing its condo pipeline — a telling signal about MF feasibility at this basis. Buyer, price and intended use are all unknown. CORRECTION: the "$5.0M CBRE asking price" we previously carried could NOT be verified — the live listing is unpriced. Commencement clock very likely stale (2.5+ years, no permit).</t>
         </is>
       </c>
       <c r="H22" s="37" t="inlineStr">
@@ -8571,9 +8606,9 @@
         </is>
       </c>
       <c r="F25" s="37" t="n"/>
-      <c r="G25" s="37" t="inlineStr">
-        <is>
-          <t>DEEP-DIVE VERIFIED 7/16/2026 (all verdicts survived 3-lens adversarial check). Fully entitled (council Sep 2024; DRH24-00090 refined 174→162u per city Aug 2025 Development Trends). Hawkins closed land Oct 2024, CDs complete Apr 2026, live $12.4M LP equity raise targeting Q3 2026 start. OM schedule: building permit ESTIMATED TO ISSUE ~7/21/2026; first CofO Aug 2027, last Apr 2028; 20u/mo lease-up =&gt; ~Q1 2028 first meaningful units. No permit in city lists through 6/30/2026 — stays PROPOSED. RE-CHECK Aug-Sep 2026: likely UC promotion if the raise closes. Capitalization is the timing risk. Land-use site 177 / parcel S1124223215 — conditional R-2 path being exercised.</t>
+      <c r="G25" s="93" t="inlineStr">
+        <is>
+          <t>Hawkins Companies (Boise; delivered Canyon Ridge 287u and Denton in 2025). 174u approved by Boise Council 9/10/2024 over a P&amp;Z denial recommendation (3-2 vote); 162u per the later Design Review DRH24-00090 redesign — carry 162, footnote 174. ~4.2 of 6.1 ac cleared/graded = more physical progress than any other unpermitted deal in the ring. RISK: commencement appears to expire ~9/10/2026, no extension found; 1.9 ac of the site still improved/occupied; the 3-2 approval means re-entitlement would be contested.</t>
         </is>
       </c>
       <c r="H25" s="37" t="inlineStr">
@@ -8604,9 +8639,9 @@
         </is>
       </c>
       <c r="F26" s="37" t="n"/>
-      <c r="G26" s="37" t="inlineStr">
-        <is>
-          <t>DEEP-DIVE VERIFIED 7/16/2026 (all verdicts survived 3-lens adversarial check). Annexation + rezone + DA approved 5-1 on 5/19/2026 (200u over ~19.5-20k sf commercial, four 3-story bldgs; up from the 184u resubmittal after the 2024 denial). DA recording + CZC/design review still ahead of permits =&gt; vertical realistically late 2026 at earliest, first units unlikely before late 2028 (~Q1 2029). Old LoopNet land listing inactive (assemblage complete); 7 of 10 adjacent owners gave letters of intent to sell. Keep PROPOSED — live pipeline.</t>
+      <c r="G26" s="93" t="inlineStr">
+        <is>
+          <t>Assemble Management (California-based; applicant of record David Ruby; architect The Architects Office). 200u + ~19,517 sf ground-floor commercial in four 3-story vertically-integrated buildings (up from 184u/18,226 sf at filing). Site: 4270 + 4240 E Overland Rd + 1480/1520/1560 Rolling Hill Dr, 8.16 ac, NE corner Overland &amp; S Rolling Hill Dr, ~1.0 mi from subject. Annexation + rezone (R1 to C-C) + DA approved by Council 5-1 on 5/19/2026 (H-2025-0040) OVER a unanimous P&amp;Z denial recommendation AND a staff denial recommendation. History: the original 154u plan was denied in 2024 over a mid-footprint holdout parcel. RISK: land was under LOI, not closed, at approval; the View Circle/Movado collector road is unfunded and staff warned it "may never be constructed"; single unsignalized right-in/right-out access for 200 units.</t>
         </is>
       </c>
       <c r="H26" s="37" t="inlineStr">
@@ -8633,9 +8668,9 @@
         </is>
       </c>
       <c r="F27" s="37" t="n"/>
-      <c r="G27" s="37" t="inlineStr">
-        <is>
-          <t>DEEP-DIVE VERIFIED 7/16/2026 (all verdicts survived 3-lens adversarial check). CUP H-2024-0071 live (approved 10/21/2025; commencement clock to ~Oct 2027); no appeal, foreclosure, or listing. DRB Investments says no groundbreak before 2027, townhomes first, ~$1B/900+u build-out phased 10-12 yrs. Only 2026 Pine 43 permits are SF/townhome + a monument sign — no MF permit through June 2026. Keep PROPOSED, undated; earliest plausible MF delivery ~2029. Distinct from the existing 25u 'Pine 43' comp. | AUG 2026 AUDIT: the SAME approved MDA (H-2024-0071, council 10/21/2025 4-1) also allows up to 604 vertically-integrated units + 30 TH beyond this 270u CUP — see shadow row "Pine 43 VI residential".</t>
+      <c r="G27" s="93" t="inlineStr">
+        <is>
+          <t>DRB Investments LLC (principal/co-owner Matt Baker) — built Dovetail (240u, 2020-23) inside this same master plan, so execution credibility is genuine. 270u CUP in two buildings on 6.28 ac with a height exception to 87 ft, approved by Council 4-1 on 10/21/2025; commencement runs to ~10/21/2027. E Pine Ave between Locust Grove &amp; Hickory. DISTINCT from the built Dovetail community at 1350 N Webb Way — do not conflate. SHADOW: the same MDA allows up to ~604 vertically-integrated units + ~30-35 townhomes (up to ~848-900 total apartments) plus ~218-229k sf office, a hotel/conference center and retail on 33+ ac, ~$1B, phased over 10-12 years — carried as a shadow row, not counted. RISK: developer guidance is townhomes first, groundbreaking "2027 or later"; podium/underground parking basis is well above the garden benchmark.</t>
         </is>
       </c>
       <c r="H27" s="37" t="inlineStr">
@@ -8732,9 +8767,9 @@
         </is>
       </c>
       <c r="F30" s="37" t="n"/>
-      <c r="G30" s="37" t="inlineStr">
-        <is>
-          <t>DEEP-DIVE VERIFIED 7/16/2026 (all verdicts survived 3-lens adversarial check). Tommy Ahlquist (Gray Owl Holdings) + The Pacific Companies bought the failed Union 93 block at the Ada County Sheriff's foreclosure auction Oct 2025 and on 7/13/2026 announced Heritage Square: the existing concrete skeleton repurposed into TWO residential towers totaling ~250 units + 120k sf Class A office + 32k sf retail (Babcock Design; McAlvain GC). Owners hope to start late 2026/early 2027, 20-24 mo buildout =&gt; ~Q1 2029. No permits issued yet — PROPOSED. Replaces the dead Union 93 row (dropped; see its diligence entry).</t>
+      <c r="G30" s="93" t="inlineStr">
+        <is>
+          <t>Residential by The Pacific Companies (Eagle ID; Caleb Roope); office/retail by Ahlquist (Tommy Ahlquist), title via Gray Owl Holdings. ~250u — DOWN from the 385 apartments approved under the original Union 93 CUP; flag that drop. Site: SE corner Main &amp; Broadway, downtown Meridian, across from City Hall. ENTITLEMENT: functionally unentitled for the current program — the 2020 CUP covered 385u/28,000 sf retail with no office tower or hotel; the new ~250u + 120,000 sf office + 32,000 sf retail concept has no confirmed application on file, described as "very nascent design." Predecessor Union 93 died on a $22M judgment and sheriff auction Oct 2025; spec office + hotel in the new stack is a real execution risk on a site that already consumed $20M+.</t>
         </is>
       </c>
       <c r="H30" s="37" t="inlineStr">
@@ -8749,12 +8784,11 @@
           <t>Outer Banks Apartments</t>
         </is>
       </c>
-      <c r="C32" s="87" t="n"/>
-      <c r="D32" s="87" t="n"/>
-      <c r="E32" s="87" t="n"/>
-      <c r="F32" s="87" t="n"/>
-      <c r="G32" s="87" t="n"/>
-      <c r="H32" s="88" t="n"/>
+      <c r="G32" s="94" t="inlineStr">
+        <is>
+          <t>Elk Ventures LLC (Erik Pilegaard, Truckee CA); owner entity 10 Mile Franklin LLC; GC Perryman Construction Mgmt. 516u = 364 apts + 126 flats + 26 TH on 19.34 ac R-40/C-C, SW corner Franklin &amp; Ten Mile. Council approved 12/14/2021; that CUP LAPSED ~Dec 2023 unused; re-approved unchanged as H-2024-0026 (P&amp;Z 10/3/2024). Sewer/water easement ESMT-2025-0071 approved 8/12/2025. Permits C-MULTI-2025-0023/-0024 + a third issued 6/17/2026 for tri-level Bldgs A/B/C on S Tallac Ln (~18-26 units). RISK: only 3 of ~50 buildings permitted; financing for later phases UNVERIFIED; Ten Mile LOS flagged unacceptable ~1 hr/day by staff in 2021.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="37" t="inlineStr">
@@ -8803,9 +8837,9 @@
         </is>
       </c>
       <c r="F34" s="37" t="n"/>
-      <c r="G34" s="37" t="inlineStr">
-        <is>
-          <t>PROMOTED from shadow watch Aug 2026 (user call: it is a live proposal). Quarterra "Emblem Meridian" 250 units (apartments + TH) on ~13 ac R-15, N of Eagle &amp; Victory — ex-Artisan Victory Market site (H-2022-0066 131u BTR approved 2023, never built). Formal early plans filed June 2026 per BoiseDev 6/10/26; no hearing date yet. Nearest live MF application to the subject (1.0 mi, same Eagle Rd corridor).</t>
+      <c r="G34" s="93" t="inlineStr">
+        <is>
+          <t>Quarterra — majority-owned by TPG Real Estate as of Jan 2026 (Lennar sold control, retained a minority stake; TPG committed $1B fresh capital). 250u = 204 apartments + 46 townhomes (~440 bedrooms) is the plan of record; the 256u/$78.0M/6.65-6.80% YoC figures are Quarterra's internal merchant model. Site: ~13-14 ac at the NE corner of S Eagle Rd (SH-55) &amp; E Victory Rd — the same 14.473-ac R-15 parcel as the prior "Artisan Victory Market" approval (138 BTR units, H-2022-0066, approved 2023, never built; our file said 131 — 138 is correct). CRITICAL: Quarterra does NOT own the land — June 2026 press confirms Baron Properties still owns it and is trying to sell. ENTITLEMENT: pre-application/concept only — no formal Meridian application, no H-file, no hearing scheduled. 18 u/ac requires a discretionary comp-plan amendment against a 15 u/ac cap. NOTE: we hold Quarterra's actual equity book + merchant model — see replacement_cost_analysis.md; its ancillary income runs +83% vs what the subject collects.</t>
         </is>
       </c>
       <c r="H34" s="37" t="inlineStr">
@@ -8834,9 +8868,9 @@
         </is>
       </c>
       <c r="F35" s="37" t="n"/>
-      <c r="G35" s="37" t="inlineStr">
-        <is>
-          <t>AUG 2026: Developer identified = Endurance Holdings LLC + Challenger Development Inc (Corey Barton / CBH Homes org; same family as Yellowstone #16). Filed 2022 as "Vanguard Commons" (432u: 3-story apts + 2-story TH, 760-1,690 SF); DA amendment hearings into Sept 2024; CoStar now carries 552u UC / Q1 2028 — and its whole 5-mi UC series equals this one deal (552u), implying observed construction. BUT no C-MULTI permit for 1085 S Ten Mile appears in Meridian public permit reports 2025-26 (only unrelated commercial on Vanguard Way) and no groundbreaking press. Verify with Meridian Building or site visit before relying on delivery timing.</t>
+      <c r="G35" s="93" t="inlineStr">
+        <is>
+          <t>Endurance Holdings LLC + Challenger Development Inc (Corey Barton / CBH-affiliated; DA also includes Ten Mile West Commercial LLC, all at 1977 W Overland Rd); original applicant of record Meridian 118 LLC. 552u is the entitled figure (432 was an earlier design iteration). Residential component is an unplatted 32.55-ac R-15 parcel (S1215131410, PROPCODE L, no TOTALVALUE) inside a ~115-ac mixed-use assemblage at Ten Mile &amp; I-84. CORRECTION: the CoStar UC/Q1-2028 flag is bleed-over from the $50.7M Life Time club (C-NEW-2026-0003) on a commercial lot in the same plat — zero permits on the R-15 parcel across 5 weekly + the Jan-2026 monthly permit reports. Commercial lots ARE building; the MF parcel is untouched 4 years post-approval. DA absorbed into the commercial-first District at Ten Mile agreement.</t>
         </is>
       </c>
       <c r="H35" s="37" t="inlineStr">
@@ -9779,7 +9813,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B32:H32"/>
+    <mergeCell ref="B36:H36"/>
     <mergeCell ref="B2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Reorder proposed by likelihood; renumber every bucket from 1; sync map
- Proposed sorted most-likely first (Heritage Square 38% -> 12548 W Overland 12%),
  ties broken by unit count
- Each bucket now numbers from 1: Stabilized 1-22, Leasing 1-5, UC 1-5, Proposed 1-15.
  Colour is the differentiator, per request
- S&U under-construction block relinked to the re-sorted CA rows
- Map pins renumbered to match; header/footer explain that numbers restart per bucket
  and that proposed is ordered most-likely first

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CQcHG3mGNNEuNdk4jQMCJB
</commit_message>
<xml_diff>
--- a/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
+++ b/SeasonsMeridian/Seasons at Meridian - Supply Chart.xlsx
@@ -914,7 +914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:M61"/>
+  <dimension ref="B1:M63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="79" min="1" max="1"/>
@@ -931,6 +931,7 @@
     <col hidden="1" width="13" customWidth="1" style="79" min="13" max="13"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="22.05" customHeight="1" s="79">
       <c r="C2" s="82" t="inlineStr">
         <is>
@@ -1989,7 +1990,7 @@
     </row>
     <row r="30">
       <c r="B30" s="10" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
@@ -2035,7 +2036,7 @@
     </row>
     <row r="31">
       <c r="B31" s="10" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
@@ -2081,7 +2082,7 @@
     </row>
     <row r="32">
       <c r="B32" s="10" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
@@ -2129,7 +2130,7 @@
     </row>
     <row r="33">
       <c r="B33" s="10" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
@@ -2175,7 +2176,7 @@
     </row>
     <row r="34">
       <c r="B34" s="10" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
@@ -2232,7 +2233,7 @@
     </row>
     <row r="37">
       <c r="B37" s="17" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="C37" s="18" t="inlineStr">
         <is>
@@ -2278,7 +2279,7 @@
     </row>
     <row r="38">
       <c r="B38" s="17" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="C38" s="18" t="inlineStr">
         <is>
@@ -2320,7 +2321,7 @@
     </row>
     <row r="39">
       <c r="B39" s="17" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="C39" s="18" t="inlineStr">
         <is>
@@ -2362,7 +2363,7 @@
     </row>
     <row r="40">
       <c r="B40" s="17" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="C40" s="18" t="inlineStr">
         <is>
@@ -2408,7 +2409,7 @@
     </row>
     <row r="41">
       <c r="B41" s="17" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
@@ -2462,19 +2463,19 @@
     </row>
     <row r="44">
       <c r="B44" s="24" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="C44" s="25" t="inlineStr">
         <is>
-          <t>Vanguard Village</t>
+          <t>Heritage Square (ex-Union 93)</t>
         </is>
       </c>
       <c r="D44" s="26" t="n">
-        <v>552</v>
+        <v>250</v>
       </c>
       <c r="E44" s="24" t="inlineStr">
         <is>
-          <t>Q1 2028</t>
+          <t>Q1 2029</t>
         </is>
       </c>
       <c r="F44" s="27" t="n"/>
@@ -2485,24 +2486,20 @@
       </c>
       <c r="H44" s="92" t="inlineStr">
         <is>
-          <t>Endurance Holdings / Challenger Dev (CBH)</t>
+          <t>Pacific Companies + Ahlquist (Gray Owl)</t>
         </is>
       </c>
       <c r="I44" s="29" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J44" s="24" t="inlineStr">
-        <is>
-          <t>Mid-Rise</t>
-        </is>
-      </c>
+        <v>1.9</v>
+      </c>
+      <c r="J44" s="24" t="n"/>
       <c r="K44" s="92" t="inlineStr">
         <is>
-          <t>NOT under construction — CoStar flag is wrong. Raw land, zero permits, CUP likely lapsed ~Jul 2024. Treat as dormant paper.</t>
+          <t>Strong sponsors and a cheap basis ($6.77M at foreclosure) — but NO application filed as of Aug 2026 and the program is unentitled. 2030 at best.</t>
         </is>
       </c>
       <c r="L44" s="90" t="n">
-        <v>0.12</v>
+        <v>0.38</v>
       </c>
       <c r="M44">
         <f>IFERROR(VALUE(RIGHT(E44,4))*4+MATCH(LEFT(E44,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
@@ -2511,19 +2508,19 @@
     </row>
     <row r="45">
       <c r="B45" s="24" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="C45" s="25" t="inlineStr">
         <is>
-          <t>The Judy (Maple Grove &amp; Overland)</t>
+          <t>Rolling Hill (Assemble Management)</t>
         </is>
       </c>
       <c r="D45" s="26" t="n">
-        <v>162</v>
+        <v>200</v>
       </c>
       <c r="E45" s="24" t="inlineStr">
         <is>
-          <t>Q1 2028</t>
+          <t>Q1 2029</t>
         </is>
       </c>
       <c r="F45" s="27" t="n"/>
@@ -2534,20 +2531,20 @@
       </c>
       <c r="H45" s="92" t="inlineStr">
         <is>
-          <t>Hawkins Companies</t>
+          <t>Assemble Management</t>
         </is>
       </c>
       <c r="I45" s="29" t="n">
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="J45" s="24" t="n"/>
       <c r="K45" s="92" t="inlineStr">
         <is>
-          <t>Real dirt moved (~4.2 of 6.1 ac graded) but the CUP clock appears to expire ~9/10/26 with no extension found. Watch for a lapse or extension filing.</t>
+          <t>Freshest entitlement in the ring (approved 5-1 on 5/19/26, no lapse risk to ~2028) — but land was LOI-stage, not closed, and the access road is unfunded.</t>
         </is>
       </c>
       <c r="L45" s="90" t="n">
-        <v>0.25</v>
+        <v>0.32</v>
       </c>
       <c r="M45">
         <f>IFERROR(VALUE(RIGHT(E45,4))*4+MATCH(LEFT(E45,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
@@ -2556,19 +2553,19 @@
     </row>
     <row r="46">
       <c r="B46" s="24" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="C46" s="25" t="inlineStr">
         <is>
-          <t>Heritage Square (ex-Union 93)</t>
+          <t>Pine 43 Multifamily (H-2024-0071 CUP)</t>
         </is>
       </c>
       <c r="D46" s="26" t="n">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="E46" s="24" t="inlineStr">
         <is>
-          <t>Q1 2029</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="F46" s="27" t="n"/>
@@ -2579,20 +2576,20 @@
       </c>
       <c r="H46" s="92" t="inlineStr">
         <is>
-          <t>Pacific Companies + Ahlquist (Gray Owl)</t>
+          <t>DRB Investments (Matt Baker)</t>
         </is>
       </c>
       <c r="I46" s="29" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
       <c r="J46" s="24" t="n"/>
       <c r="K46" s="92" t="inlineStr">
         <is>
-          <t>Strong sponsors and a cheap basis ($6.77M at foreclosure) — but NO application filed as of Aug 2026 and the program is unentitled. 2030 at best.</t>
+          <t>CUP current to ~10/21/27 and the sponsor has real credibility (built Dovetail here) — but its own guidance is townhomes FIRST, groundbreaking "2027 or later."</t>
         </is>
       </c>
       <c r="L46" s="90" t="n">
-        <v>0.38</v>
+        <v>0.3</v>
       </c>
       <c r="M46">
         <f>IFERROR(VALUE(RIGHT(E46,4))*4+MATCH(LEFT(E46,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
@@ -2601,19 +2598,19 @@
     </row>
     <row r="47">
       <c r="B47" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C47" s="25" t="inlineStr">
+        <is>
+          <t>Meridian OZ Apartments</t>
+        </is>
+      </c>
+      <c r="D47" s="26" t="n">
         <v>36</v>
       </c>
-      <c r="C47" s="25" t="inlineStr">
-        <is>
-          <t>The Cole Denton</t>
-        </is>
-      </c>
-      <c r="D47" s="26" t="n">
-        <v>224</v>
-      </c>
       <c r="E47" s="24" t="inlineStr">
         <is>
-          <t>Q1 2029</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="F47" s="27" t="n"/>
@@ -2624,24 +2621,24 @@
       </c>
       <c r="H47" s="92" t="inlineStr">
         <is>
-          <t>Kal Pacific (Don Veasy)</t>
+          <t>SOLD 8/7/26 — buyer unknown (was Realm Venture)</t>
         </is>
       </c>
       <c r="I47" s="29" t="n">
-        <v>4.5</v>
+        <v>1.1</v>
       </c>
       <c r="J47" s="24" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K47" s="92" t="inlineStr">
         <is>
-          <t>No entitlement for the 224u program — the only approval this site ever had was a 2021 DA for 136u that was never permitted. Post-2031.</t>
+          <t>SOLD 8/7/26 for $1.7M. CUP expires ~10/17/26 — about 8 weeks out — with no extension filed and no sign the new owner is moving to permit.</t>
         </is>
       </c>
       <c r="L47" s="90" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="M47">
         <f>IFERROR(VALUE(RIGHT(E47,4))*4+MATCH(LEFT(E47,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
@@ -2650,19 +2647,19 @@
     </row>
     <row r="48">
       <c r="B48" s="24" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C48" s="25" t="inlineStr">
         <is>
-          <t>Rolling Hill (Assemble Management)</t>
+          <t>12565 West Fairview Avenue</t>
         </is>
       </c>
       <c r="D48" s="26" t="n">
-        <v>200</v>
+        <v>275</v>
       </c>
       <c r="E48" s="24" t="inlineStr">
         <is>
-          <t>Q1 2029</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="F48" s="27" t="n"/>
@@ -2673,20 +2670,24 @@
       </c>
       <c r="H48" s="92" t="inlineStr">
         <is>
-          <t>Assemble Management</t>
+          <t>UNVERIFIED — not publicly disclosed</t>
         </is>
       </c>
       <c r="I48" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="J48" s="24" t="n"/>
+        <v>2.1</v>
+      </c>
+      <c r="J48" s="24" t="inlineStr">
+        <is>
+          <t>Mid-Rise</t>
+        </is>
+      </c>
       <c r="K48" s="92" t="inlineStr">
         <is>
-          <t>Freshest entitlement in the ring (approved 5-1 on 5/19/26, no lapse risk to ~2028) — but land was LOI-stage, not closed, and the access road is unfunded.</t>
+          <t>Shows "Entitled" on Boise's tracker but the developer is unknown and there is no permit 16 months post concept review. Structured-parking product needs rents well above the garden hurdle.</t>
         </is>
       </c>
       <c r="L48" s="90" t="n">
-        <v>0.32</v>
+        <v>0.25</v>
       </c>
       <c r="M48">
         <f>IFERROR(VALUE(RIGHT(E48,4))*4+MATCH(LEFT(E48,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
@@ -2695,19 +2696,19 @@
     </row>
     <row r="49">
       <c r="B49" s="24" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C49" s="25" t="inlineStr">
         <is>
-          <t>Record</t>
+          <t>The Judy (Maple Grove &amp; Overland)</t>
         </is>
       </c>
       <c r="D49" s="26" t="n">
-        <v>472</v>
+        <v>162</v>
       </c>
       <c r="E49" s="24" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Q1 2028</t>
         </is>
       </c>
       <c r="F49" s="27" t="n"/>
@@ -2718,24 +2719,20 @@
       </c>
       <c r="H49" s="92" t="inlineStr">
         <is>
-          <t>Brighton Development</t>
+          <t>Hawkins Companies</t>
         </is>
       </c>
       <c r="I49" s="29" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="J49" s="24" t="inlineStr">
-        <is>
-          <t>Mid-Rise</t>
-        </is>
-      </c>
+        <v>3.4</v>
+      </c>
+      <c r="J49" s="24" t="n"/>
       <c r="K49" s="92" t="inlineStr">
         <is>
-          <t>ENTITLEMENT LAPSED. Base clock ran out ~Apr/May 2024 and even a maximum extension expired ~Apr/May 2026. Requires full re-entitlement.</t>
+          <t>Real dirt moved (~4.2 of 6.1 ac graded) but the CUP clock appears to expire ~9/10/26 with no extension found. Watch for a lapse or extension filing.</t>
         </is>
       </c>
       <c r="L49" s="90" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="M49">
         <f>IFERROR(VALUE(RIGHT(E49,4))*4+MATCH(LEFT(E49,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
@@ -2744,15 +2741,15 @@
     </row>
     <row r="50">
       <c r="B50" s="24" t="n">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="C50" s="25" t="inlineStr">
         <is>
-          <t>The Gateway at Ten Mile</t>
+          <t>Ascent Overland</t>
         </is>
       </c>
       <c r="D50" s="26" t="n">
-        <v>390</v>
+        <v>138</v>
       </c>
       <c r="E50" s="24" t="inlineStr">
         <is>
@@ -2767,11 +2764,11 @@
       </c>
       <c r="H50" s="92" t="inlineStr">
         <is>
-          <t>GFI Meridian Investments (Trevor Gasser)</t>
+          <t>MVRK Development (under contract 8/7/26)</t>
         </is>
       </c>
       <c r="I50" s="29" t="n">
-        <v>3.7</v>
+        <v>1.5</v>
       </c>
       <c r="J50" s="24" t="inlineStr">
         <is>
@@ -2780,11 +2777,11 @@
       </c>
       <c r="K50" s="92" t="inlineStr">
         <is>
-          <t>Developer says residential is 5-7 years out; commercial builds first and is only at pad-leasing stage. CUP lapses ~11/19/26.</t>
+          <t>UNDER CONTRACT 8/7/26 after 469 days on market — the developer chose to sell rather than build. Buyer and intent unknown.</t>
         </is>
       </c>
       <c r="L50" s="90" t="n">
-        <v>0.15</v>
+        <v>0.22</v>
       </c>
       <c r="M50">
         <f>IFERROR(VALUE(RIGHT(E50,4))*4+MATCH(LEFT(E50,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
@@ -2793,15 +2790,15 @@
     </row>
     <row r="51">
       <c r="B51" s="24" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="C51" s="25" t="inlineStr">
         <is>
-          <t>Syringa Crossing</t>
+          <t>Record</t>
         </is>
       </c>
       <c r="D51" s="26" t="n">
-        <v>302</v>
+        <v>472</v>
       </c>
       <c r="E51" s="24" t="inlineStr">
         <is>
@@ -2816,11 +2813,11 @@
       </c>
       <c r="H51" s="92" t="inlineStr">
         <is>
-          <t>Hawkins Companies</t>
+          <t>Brighton Development</t>
         </is>
       </c>
       <c r="I51" s="29" t="n">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
       <c r="J51" s="24" t="inlineStr">
         <is>
@@ -2829,11 +2826,11 @@
       </c>
       <c r="K51" s="92" t="inlineStr">
         <is>
-          <t>NOT entitled. Unanimous P&amp;Z denial rec 4/2/26, council remand 6/16/26, re-heard 8/6/26 with the outcome still unpublished. 302u is Phase 1 only.</t>
+          <t>ENTITLEMENT LAPSED. Base clock ran out ~Apr/May 2024 and even a maximum extension expired ~Apr/May 2026. Requires full re-entitlement.</t>
         </is>
       </c>
       <c r="L51" s="90" t="n">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="M51">
         <f>IFERROR(VALUE(RIGHT(E51,4))*4+MATCH(LEFT(E51,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
@@ -2842,7 +2839,7 @@
     </row>
     <row r="52">
       <c r="B52" s="24" t="n">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C52" s="25" t="inlineStr">
         <is>
@@ -2891,15 +2888,15 @@
     </row>
     <row r="53">
       <c r="B53" s="24" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="C53" s="25" t="inlineStr">
         <is>
-          <t>12565 West Fairview Avenue</t>
+          <t>Emblem Meridian (Quarterra)</t>
         </is>
       </c>
       <c r="D53" s="26" t="n">
-        <v>275</v>
+        <v>250</v>
       </c>
       <c r="E53" s="24" t="inlineStr">
         <is>
@@ -2914,24 +2911,24 @@
       </c>
       <c r="H53" s="92" t="inlineStr">
         <is>
-          <t>UNVERIFIED — not publicly disclosed</t>
+          <t>Quarterra (TPG-controlled); land: Baron Properties</t>
         </is>
       </c>
       <c r="I53" s="29" t="n">
-        <v>2.1</v>
+        <v>1</v>
       </c>
       <c r="J53" s="24" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K53" s="92" t="inlineStr">
         <is>
-          <t>Shows "Entitled" on Boise's tracker but the developer is unknown and there is no permit 16 months post concept review. Structured-parking product needs rents well above the garden hurdle.</t>
+          <t>Earliest-stage deal in the pipeline — no application, no H-file, no hearing, AND Quarterra does not own the land (Baron is still trying to sell it).</t>
         </is>
       </c>
       <c r="L53" s="90" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="M53">
         <f>IFERROR(VALUE(RIGHT(E53,4))*4+MATCH(LEFT(E53,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
@@ -2940,15 +2937,15 @@
     </row>
     <row r="54">
       <c r="B54" s="24" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="C54" s="25" t="inlineStr">
         <is>
-          <t>Pine 43 Multifamily (H-2024-0071 CUP)</t>
+          <t>The Gateway at Ten Mile</t>
         </is>
       </c>
       <c r="D54" s="26" t="n">
-        <v>270</v>
+        <v>390</v>
       </c>
       <c r="E54" s="24" t="inlineStr">
         <is>
@@ -2963,20 +2960,24 @@
       </c>
       <c r="H54" s="92" t="inlineStr">
         <is>
-          <t>DRB Investments (Matt Baker)</t>
+          <t>GFI Meridian Investments (Trevor Gasser)</t>
         </is>
       </c>
       <c r="I54" s="29" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="J54" s="24" t="n"/>
+        <v>3.7</v>
+      </c>
+      <c r="J54" s="24" t="inlineStr">
+        <is>
+          <t>Mid-Rise</t>
+        </is>
+      </c>
       <c r="K54" s="92" t="inlineStr">
         <is>
-          <t>CUP current to ~10/21/27 and the sponsor has real credibility (built Dovetail here) — but its own guidance is townhomes FIRST, groundbreaking "2027 or later."</t>
+          <t>Developer says residential is 5-7 years out; commercial builds first and is only at pad-leasing stage. CUP lapses ~11/19/26.</t>
         </is>
       </c>
       <c r="L54" s="90" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="M54">
         <f>IFERROR(VALUE(RIGHT(E54,4))*4+MATCH(LEFT(E54,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
@@ -2985,19 +2986,19 @@
     </row>
     <row r="55">
       <c r="B55" s="24" t="n">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C55" s="25" t="inlineStr">
         <is>
-          <t>Emblem Meridian (Quarterra)</t>
+          <t>The Cole Denton</t>
         </is>
       </c>
       <c r="D55" s="26" t="n">
-        <v>250</v>
+        <v>224</v>
       </c>
       <c r="E55" s="24" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Q1 2029</t>
         </is>
       </c>
       <c r="F55" s="27" t="n"/>
@@ -3008,24 +3009,24 @@
       </c>
       <c r="H55" s="92" t="inlineStr">
         <is>
-          <t>Quarterra (TPG-controlled); land: Baron Properties</t>
+          <t>Kal Pacific (Don Veasy)</t>
         </is>
       </c>
       <c r="I55" s="29" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="J55" s="24" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K55" s="92" t="inlineStr">
         <is>
-          <t>Earliest-stage deal in the pipeline — no application, no H-file, no hearing, AND Quarterra does not own the land (Baron is still trying to sell it).</t>
+          <t>No entitlement for the 224u program — the only approval this site ever had was a 2021 DA for 136u that was never permitted. Post-2031.</t>
         </is>
       </c>
       <c r="L55" s="90" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="M55">
         <f>IFERROR(VALUE(RIGHT(E55,4))*4+MATCH(LEFT(E55,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
@@ -3034,19 +3035,19 @@
     </row>
     <row r="56">
       <c r="B56" s="24" t="n">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C56" s="25" t="inlineStr">
         <is>
-          <t>12548 West Overland Road</t>
+          <t>Vanguard Village</t>
         </is>
       </c>
       <c r="D56" s="26" t="n">
-        <v>156</v>
+        <v>552</v>
       </c>
       <c r="E56" s="24" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Q1 2028</t>
         </is>
       </c>
       <c r="F56" s="27" t="n"/>
@@ -3057,11 +3058,11 @@
       </c>
       <c r="H56" s="92" t="inlineStr">
         <is>
-          <t>Hook Family Trust</t>
+          <t>Endurance Holdings / Challenger Dev (CBH)</t>
         </is>
       </c>
       <c r="I56" s="29" t="n">
-        <v>1.1</v>
+        <v>4.3</v>
       </c>
       <c r="J56" s="24" t="inlineStr">
         <is>
@@ -3070,7 +3071,7 @@
       </c>
       <c r="K56" s="92" t="inlineStr">
         <is>
-          <t>LAPSED — PUD commencement passed ~3/12/26 with no extension ever filed; zero city activity since 10/23/23. Site earns income as RV storage.</t>
+          <t>NOT under construction — CoStar flag is wrong. Raw land, zero permits, CUP likely lapsed ~Jul 2024. Treat as dormant paper.</t>
         </is>
       </c>
       <c r="L56" s="90" t="n">
@@ -3083,15 +3084,15 @@
     </row>
     <row r="57">
       <c r="B57" s="24" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="C57" s="25" t="inlineStr">
         <is>
-          <t>Ascent Overland</t>
+          <t>Syringa Crossing</t>
         </is>
       </c>
       <c r="D57" s="26" t="n">
-        <v>138</v>
+        <v>302</v>
       </c>
       <c r="E57" s="24" t="inlineStr">
         <is>
@@ -3106,11 +3107,11 @@
       </c>
       <c r="H57" s="92" t="inlineStr">
         <is>
-          <t>MVRK Development (under contract 8/7/26)</t>
+          <t>Hawkins Companies</t>
         </is>
       </c>
       <c r="I57" s="29" t="n">
-        <v>1.5</v>
+        <v>2.8</v>
       </c>
       <c r="J57" s="24" t="inlineStr">
         <is>
@@ -3119,11 +3120,11 @@
       </c>
       <c r="K57" s="92" t="inlineStr">
         <is>
-          <t>UNDER CONTRACT 8/7/26 after 469 days on market — the developer chose to sell rather than build. Buyer and intent unknown.</t>
+          <t>NOT entitled. Unanimous P&amp;Z denial rec 4/2/26, council remand 6/16/26, re-heard 8/6/26 with the outcome still unpublished. 302u is Phase 1 only.</t>
         </is>
       </c>
       <c r="L57" s="90" t="n">
-        <v>0.22</v>
+        <v>0.12</v>
       </c>
       <c r="M57">
         <f>IFERROR(VALUE(RIGHT(E57,4))*4+MATCH(LEFT(E57,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
@@ -3132,15 +3133,15 @@
     </row>
     <row r="58">
       <c r="B58" s="24" t="n">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="C58" s="25" t="inlineStr">
         <is>
-          <t>Meridian OZ Apartments</t>
+          <t>12548 West Overland Road</t>
         </is>
       </c>
       <c r="D58" s="26" t="n">
-        <v>36</v>
+        <v>156</v>
       </c>
       <c r="E58" s="24" t="inlineStr">
         <is>
@@ -3155,7 +3156,7 @@
       </c>
       <c r="H58" s="92" t="inlineStr">
         <is>
-          <t>SOLD 8/7/26 — buyer unknown (was Realm Venture)</t>
+          <t>Hook Family Trust</t>
         </is>
       </c>
       <c r="I58" s="29" t="n">
@@ -3163,16 +3164,16 @@
       </c>
       <c r="J58" s="24" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K58" s="92" t="inlineStr">
         <is>
-          <t>SOLD 8/7/26 for $1.7M. CUP expires ~10/17/26 — about 8 weeks out — with no extension filed and no sign the new owner is moving to permit.</t>
+          <t>LAPSED — PUD commencement passed ~3/12/26 with no extension ever filed; zero city activity since 10/23/23. Site earns income as RV storage.</t>
         </is>
       </c>
       <c r="L58" s="90" t="n">
-        <v>0.3</v>
+        <v>0.12</v>
       </c>
       <c r="M58">
         <f>IFERROR(VALUE(RIGHT(E58,4))*4+MATCH(LEFT(E58,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
@@ -3188,6 +3189,8 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
+    <row r="63"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="B3:G3"/>
@@ -3299,15 +3302,15 @@
         </is>
       </c>
       <c r="R5" s="37">
-        <f>'Competitive Analysis'!C40</f>
+        <f>'Competitive Analysis'!C37</f>
         <v/>
       </c>
       <c r="S5" s="38">
-        <f>'Competitive Analysis'!D40</f>
+        <f>'Competitive Analysis'!D37</f>
         <v/>
       </c>
       <c r="T5" s="39">
-        <f>'Competitive Analysis'!E40</f>
+        <f>'Competitive Analysis'!E37</f>
         <v/>
       </c>
       <c r="V5">
@@ -3329,15 +3332,15 @@
         <v>0.95</v>
       </c>
       <c r="R6" s="37">
-        <f>'Competitive Analysis'!C37</f>
+        <f>'Competitive Analysis'!C38</f>
         <v/>
       </c>
       <c r="S6" s="38">
-        <f>'Competitive Analysis'!D37</f>
+        <f>'Competitive Analysis'!D38</f>
         <v/>
       </c>
       <c r="T6" s="39">
-        <f>'Competitive Analysis'!E37</f>
+        <f>'Competitive Analysis'!E38</f>
         <v/>
       </c>
       <c r="V6">
@@ -3361,15 +3364,15 @@
         </is>
       </c>
       <c r="R7" s="37">
-        <f>'Competitive Analysis'!C38</f>
+        <f>'Competitive Analysis'!C39</f>
         <v/>
       </c>
       <c r="S7" s="38">
-        <f>'Competitive Analysis'!D38</f>
+        <f>'Competitive Analysis'!D39</f>
         <v/>
       </c>
       <c r="T7" s="39">
-        <f>'Competitive Analysis'!E38</f>
+        <f>'Competitive Analysis'!E39</f>
         <v/>
       </c>
       <c r="V7">
@@ -3391,15 +3394,15 @@
         <v>425</v>
       </c>
       <c r="R8" s="37">
-        <f>'Competitive Analysis'!C39</f>
+        <f>'Competitive Analysis'!C40</f>
         <v/>
       </c>
       <c r="S8" s="38">
-        <f>'Competitive Analysis'!D39</f>
+        <f>'Competitive Analysis'!D40</f>
         <v/>
       </c>
       <c r="T8" s="39">
-        <f>'Competitive Analysis'!E39</f>
+        <f>'Competitive Analysis'!E40</f>
         <v/>
       </c>
       <c r="V8">

</xml_diff>